<commit_message>
complete with storage const
</commit_message>
<xml_diff>
--- a/WithCapacityConst.xlsx
+++ b/WithCapacityConst.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/debdeeppaul/Documents/Procurement/PIDSG25/pricesaa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CC41115-32F7-A244-B5A2-E7FF5DF85A6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7F47193-BA8F-9F4E-BC08-99477A2A4F7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5980" yWindow="3940" windowWidth="16380" windowHeight="12220" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4580" yWindow="3500" windowWidth="19420" windowHeight="11500" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="04" sheetId="1" r:id="rId1"/>
-    <sheet name="05" sheetId="9" r:id="rId2"/>
-    <sheet name="06" sheetId="7" r:id="rId3"/>
-    <sheet name="07" sheetId="8" r:id="rId4"/>
-    <sheet name="08" sheetId="6" r:id="rId5"/>
+    <sheet name="05" sheetId="10" r:id="rId2"/>
+    <sheet name="05Asol" sheetId="9" r:id="rId3"/>
+    <sheet name="06" sheetId="7" r:id="rId4"/>
+    <sheet name="07" sheetId="8" r:id="rId5"/>
+    <sheet name="08" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="22">
   <si>
     <t>Hedged price</t>
   </si>
@@ -76,6 +77,36 @@
   </si>
   <si>
     <t>AI-storage</t>
+  </si>
+  <si>
+    <t>Procurement</t>
+  </si>
+  <si>
+    <t>Storage</t>
+  </si>
+  <si>
+    <t>Backlog</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Man</t>
+  </si>
+  <si>
+    <t>Price-SAA</t>
+  </si>
+  <si>
+    <t>AI</t>
+  </si>
+  <si>
+    <t>Hed</t>
+  </si>
+  <si>
+    <t>Unhed</t>
+  </si>
+  <si>
+    <t>USD</t>
   </si>
 </sst>
 </file>
@@ -120,7 +151,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -130,6 +161,10 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -391,7 +426,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="12.6640625" customWidth="1"/>
@@ -441,10 +476,10 @@
         <v>45772</v>
       </c>
       <c r="B2">
-        <v>1.5288157894736842</v>
+        <v>47.552286315789345</v>
       </c>
       <c r="C2">
-        <v>1.4112105263157895</v>
+        <v>43.894292210526316</v>
       </c>
       <c r="D2" s="2">
         <v>4886.8312757201647</v>
@@ -459,7 +494,7 @@
       <c r="G2" s="2">
         <v>4886.8312757201647</v>
       </c>
-      <c r="H2" s="4">
+      <c r="H2">
         <v>7000</v>
       </c>
       <c r="I2">
@@ -467,14 +502,15 @@
         <v>11886.831275720164</v>
       </c>
       <c r="J2">
-        <v>5195.1035206425595</v>
+        <v>9773.6625514403295</v>
       </c>
       <c r="K2">
         <f>F2-J2</f>
-        <v>4578.55903079777</v>
+        <v>0</v>
       </c>
       <c r="L2">
-        <v>2113.1687242798298</v>
+        <f>I2-J2</f>
+        <v>2113.1687242798344</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
@@ -482,7 +518,7 @@
         <v>45802</v>
       </c>
       <c r="B3">
-        <v>1.5806907894736841</v>
+        <v>49.165806315789467</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -500,7 +536,7 @@
       <c r="G3" s="2">
         <v>4886.8312757201647</v>
       </c>
-      <c r="H3" s="4">
+      <c r="H3">
         <v>7000</v>
       </c>
       <c r="I3">
@@ -508,13 +544,14 @@
         <v>11886.831275720164</v>
       </c>
       <c r="J3">
-        <v>5907.1382972953343</v>
+        <v>5079.7325102880659</v>
       </c>
       <c r="K3">
         <f>K2+F3-J3</f>
-        <v>3751.1532437905025</v>
+        <v>0</v>
       </c>
       <c r="L3">
+        <f>L2+I3-J3</f>
         <v>8920.2674897119323</v>
       </c>
     </row>
@@ -523,10 +560,10 @@
         <v>45833</v>
       </c>
       <c r="B4">
-        <v>1.6237697368421053</v>
+        <v>50.505733894736842</v>
       </c>
       <c r="C4">
-        <v>1.4613947368421052</v>
+        <v>45.455221894736837</v>
       </c>
       <c r="D4" s="2">
         <v>4886.8312757201647</v>
@@ -541,7 +578,7 @@
       <c r="G4" s="2">
         <v>4886.8312757201647</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4">
         <v>7000</v>
       </c>
       <c r="I4">
@@ -549,13 +586,14 @@
         <v>11886.831275720164</v>
       </c>
       <c r="J4">
-        <v>5625.7573205650187</v>
+        <v>9902.2633744855975</v>
       </c>
       <c r="K4">
         <f t="shared" ref="K4:K13" si="2">K3+F4-J4</f>
-        <v>8027.6592977110813</v>
+        <v>0</v>
       </c>
       <c r="L4">
+        <f>L3+I4-J4</f>
         <v>10904.835390946499</v>
       </c>
     </row>
@@ -564,10 +602,10 @@
         <v>45863</v>
       </c>
       <c r="B5">
-        <v>1.6237697368421053</v>
+        <v>50.505733894736842</v>
       </c>
       <c r="C5">
-        <v>0.97426315789473683</v>
+        <v>30.303481263157895</v>
       </c>
       <c r="D5" s="2">
         <v>4886.8312757201647</v>
@@ -582,7 +620,7 @@
       <c r="G5" s="2">
         <v>4886.8312757201647</v>
       </c>
-      <c r="H5" s="4">
+      <c r="H5">
         <v>7000</v>
       </c>
       <c r="I5">
@@ -590,13 +628,14 @@
         <v>11886.831275720164</v>
       </c>
       <c r="J5">
-        <v>6433.9826158977739</v>
+        <v>8326.9032921810704</v>
       </c>
       <c r="K5">
         <f t="shared" si="2"/>
-        <v>9920.5799739943777</v>
+        <v>0</v>
       </c>
       <c r="L5">
+        <f t="shared" ref="L5:L12" si="3">L4+I5-J5</f>
         <v>14464.763374485594</v>
       </c>
     </row>
@@ -605,10 +644,10 @@
         <v>45894</v>
       </c>
       <c r="B6">
-        <v>1.6237697368421053</v>
+        <v>50.505733894736842</v>
       </c>
       <c r="C6">
-        <v>0.97426315789473683</v>
+        <v>30.303481263157895</v>
       </c>
       <c r="D6" s="2">
         <v>4886.8312757201647</v>
@@ -623,7 +662,7 @@
       <c r="G6" s="2">
         <v>4886.8312757201647</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6">
         <v>6657.9218106995604</v>
       </c>
       <c r="I6">
@@ -631,13 +670,14 @@
         <v>11544.753086419725</v>
       </c>
       <c r="J6">
-        <v>6493.9081133646077</v>
+        <v>8326.9032921810704</v>
       </c>
       <c r="K6">
         <f t="shared" si="2"/>
-        <v>11753.575152810841</v>
+        <v>0</v>
       </c>
       <c r="L6">
+        <f t="shared" si="3"/>
         <v>17682.613168724245</v>
       </c>
     </row>
@@ -646,10 +686,10 @@
         <v>45925</v>
       </c>
       <c r="B7">
-        <v>1.6237697368421053</v>
+        <v>50.505733894736842</v>
       </c>
       <c r="C7">
-        <v>0.32475657894736842</v>
+        <v>10.101228631578946</v>
       </c>
       <c r="D7" s="2">
         <v>4886.8312757201647</v>
@@ -664,7 +704,7 @@
       <c r="G7" s="2">
         <v>4886.8312757201647</v>
       </c>
-      <c r="H7" s="4">
+      <c r="H7">
         <v>3279.3186831275698</v>
       </c>
       <c r="I7">
@@ -672,13 +712,14 @@
         <v>8166.1499588477345</v>
       </c>
       <c r="J7">
-        <v>6071.2326312903115</v>
+        <v>6237.1399176954737</v>
       </c>
       <c r="K7">
         <f t="shared" si="2"/>
-        <v>11919.482439216003</v>
+        <v>0</v>
       </c>
       <c r="L7">
+        <f t="shared" si="3"/>
         <v>19611.623209876507</v>
       </c>
     </row>
@@ -687,10 +728,10 @@
         <v>45955</v>
       </c>
       <c r="B8">
-        <v>1.7219534883720931</v>
+        <v>53.559641302325581</v>
       </c>
       <c r="C8">
-        <v>1.7219534883720931</v>
+        <v>53.559641302325581</v>
       </c>
       <c r="D8" s="2">
         <v>2764.9176954732511</v>
@@ -705,7 +746,7 @@
       <c r="G8" s="2">
         <v>2764.9176954732511</v>
       </c>
-      <c r="H8" s="4">
+      <c r="H8">
         <v>0</v>
       </c>
       <c r="I8">
@@ -713,13 +754,14 @@
         <v>2764.9176954732511</v>
       </c>
       <c r="J8">
-        <v>6403.8158313631438</v>
+        <v>5208.333333333333</v>
       </c>
       <c r="K8">
         <f t="shared" si="2"/>
-        <v>10723.999941186194</v>
+        <v>0</v>
       </c>
       <c r="L8">
+        <f t="shared" si="3"/>
         <v>17168.207572016425</v>
       </c>
     </row>
@@ -728,10 +770,10 @@
         <v>45986</v>
       </c>
       <c r="B9">
-        <v>1.720433105627585</v>
+        <v>53.512351317440405</v>
       </c>
       <c r="C9">
-        <v>1.720433105627585</v>
+        <v>53.512351317440405</v>
       </c>
       <c r="D9" s="2">
         <v>2767.3611111111113</v>
@@ -746,7 +788,7 @@
       <c r="G9" s="2">
         <v>2767.3611111111113</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9">
         <v>0</v>
       </c>
       <c r="I9">
@@ -754,13 +796,14 @@
         <v>2767.3611111111113</v>
       </c>
       <c r="J9">
-        <v>6026.4848889003415</v>
+        <v>6237.1399176954737</v>
       </c>
       <c r="K9">
         <f t="shared" si="2"/>
-        <v>10934.654969981326</v>
+        <v>0</v>
       </c>
       <c r="L9">
+        <f t="shared" si="3"/>
         <v>13698.428765432065</v>
       </c>
     </row>
@@ -769,10 +812,10 @@
         <v>46016</v>
       </c>
       <c r="B10">
-        <v>1.720433105627585</v>
+        <v>53.512351317440405</v>
       </c>
       <c r="C10">
-        <v>2.2939030624099632</v>
+        <v>71.349560853199492</v>
       </c>
       <c r="D10" s="2">
         <v>2767.3611111111113</v>
@@ -787,7 +830,7 @@
       <c r="G10" s="2">
         <v>2767.3611111111113</v>
       </c>
-      <c r="H10" s="4">
+      <c r="H10">
         <v>0</v>
       </c>
       <c r="I10">
@@ -795,13 +838,14 @@
         <v>2767.3611111111113</v>
       </c>
       <c r="J10">
-        <v>4479.7985738060161</v>
+        <v>7298.0967078189306</v>
       </c>
       <c r="K10">
         <f t="shared" si="2"/>
-        <v>13752.953103994241</v>
+        <v>0</v>
       </c>
       <c r="L10">
+        <f t="shared" si="3"/>
         <v>9167.6931687242432</v>
       </c>
     </row>
@@ -810,10 +854,10 @@
         <v>46047</v>
       </c>
       <c r="B11">
-        <v>1.720433105627585</v>
+        <v>53.512351317440405</v>
       </c>
       <c r="C11">
-        <v>0.28673497839118917</v>
+        <v>8.9186047678795468</v>
       </c>
       <c r="D11" s="2">
         <v>2767.3611111111113</v>
@@ -828,7 +872,7 @@
       <c r="G11" s="2">
         <v>2767.3611111111113</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H11">
         <v>0</v>
       </c>
       <c r="I11">
@@ -836,13 +880,14 @@
         <v>2767.3611111111113</v>
       </c>
       <c r="J11">
-        <v>4284.164832400751</v>
+        <v>3632.9732510288068</v>
       </c>
       <c r="K11">
         <f t="shared" si="2"/>
-        <v>13101.761522622295</v>
+        <v>0</v>
       </c>
       <c r="L11">
+        <f t="shared" si="3"/>
         <v>8302.0810288065477</v>
       </c>
     </row>
@@ -851,10 +896,10 @@
         <v>46078</v>
       </c>
       <c r="B12">
-        <v>1.720433105627585</v>
+        <v>53.512351317440405</v>
       </c>
       <c r="C12">
-        <v>1.4336865095961708</v>
+        <v>44.593385194479296</v>
       </c>
       <c r="D12" s="2">
         <v>2767.3611111111113</v>
@@ -869,7 +914,7 @@
       <c r="G12" s="2">
         <v>2767.3611111111113</v>
       </c>
-      <c r="H12" s="4">
+      <c r="H12">
         <v>0</v>
       </c>
       <c r="I12">
@@ -877,13 +922,14 @@
         <v>2767.3611111111113</v>
       </c>
       <c r="J12">
-        <v>3874.8158713185621</v>
+        <v>5722.7366255144034</v>
       </c>
       <c r="K12">
         <f t="shared" si="2"/>
-        <v>14949.682276818137</v>
+        <v>0</v>
       </c>
       <c r="L12">
+        <f t="shared" si="3"/>
         <v>5346.7055144032556</v>
       </c>
     </row>
@@ -892,10 +938,10 @@
         <v>46106</v>
       </c>
       <c r="B13">
-        <v>1.720433105627585</v>
+        <v>53.512351317440405</v>
       </c>
       <c r="C13">
-        <v>1.1469515312049816</v>
+        <v>35.674780426599746</v>
       </c>
       <c r="D13" s="2">
         <v>2767.3611111111113</v>
@@ -910,7 +956,7 @@
       <c r="G13" s="2">
         <v>2767.3611111111113</v>
       </c>
-      <c r="H13" s="4">
+      <c r="H13">
         <v>0</v>
       </c>
       <c r="I13">
@@ -918,14 +964,369 @@
         <v>2767.3611111111113</v>
       </c>
       <c r="J13">
-        <v>3826.840185484803</v>
+        <v>5208.333333333333</v>
       </c>
       <c r="K13">
         <f t="shared" si="2"/>
-        <v>16331.175424666666</v>
+        <v>0</v>
       </c>
       <c r="L13">
+        <f>L12+I13-J13</f>
         <v>2905.7332921810339</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B15">
+        <f>B2*31.104</f>
+        <v>1479.0663135663117</v>
+      </c>
+      <c r="C15">
+        <f>C2*31.104</f>
+        <v>1365.2880649162105</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B16">
+        <f t="shared" ref="B16:C16" si="4">B3*31.104</f>
+        <v>1529.2532396463155</v>
+      </c>
+      <c r="C16">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F16" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B17">
+        <f t="shared" ref="B17:C17" si="5">B4*31.104</f>
+        <v>1570.9303470618947</v>
+      </c>
+      <c r="C17">
+        <f t="shared" si="5"/>
+        <v>1413.8392218138945</v>
+      </c>
+      <c r="F17">
+        <f>B2*D2+C2*E2</f>
+        <v>446883.99999999942</v>
+      </c>
+      <c r="G17">
+        <f>B2*G2+C2*H2</f>
+        <v>539640.04547368363</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B18">
+        <f t="shared" ref="B18:C18" si="6">B5*31.104</f>
+        <v>1570.9303470618947</v>
+      </c>
+      <c r="C18">
+        <f t="shared" si="6"/>
+        <v>942.55948120926314</v>
+      </c>
+      <c r="F18">
+        <f t="shared" ref="F18:F28" si="7">B3*D3+C3*E3</f>
+        <v>240264.99999999997</v>
+      </c>
+      <c r="G18">
+        <f t="shared" ref="G18:G28" si="8">B3*G3+C3*H3</f>
+        <v>240264.99999999997</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B19">
+        <f t="shared" ref="B19:C19" si="9">B6*31.104</f>
+        <v>1570.9303470618947</v>
+      </c>
+      <c r="C19">
+        <f t="shared" si="9"/>
+        <v>942.55948120926314</v>
+      </c>
+      <c r="F19">
+        <f t="shared" si="7"/>
+        <v>474790.57894736843</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="8"/>
+        <v>564999.55326315784</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B20">
+        <f t="shared" ref="B20:C20" si="10">B7*31.104</f>
+        <v>1570.9303470618947</v>
+      </c>
+      <c r="C20">
+        <f t="shared" si="10"/>
+        <v>314.18861535663154</v>
+      </c>
+      <c r="F20">
+        <f t="shared" si="7"/>
+        <v>351059.15789473685</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="8"/>
+        <v>458937.36884210526</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B21">
+        <f t="shared" ref="B21:C21" si="11">B8*31.104</f>
+        <v>1665.9190830675348</v>
+      </c>
+      <c r="C21">
+        <f t="shared" si="11"/>
+        <v>1665.9190830675348</v>
+      </c>
+      <c r="F21">
+        <f t="shared" si="7"/>
+        <v>351059.15789473685</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="8"/>
+        <v>448571.20884210442</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B22">
+        <f t="shared" ref="B22:C22" si="12">B9*31.104</f>
+        <v>1664.4481753776663</v>
+      </c>
+      <c r="C22">
+        <f t="shared" si="12"/>
+        <v>1664.4481753776663</v>
+      </c>
+      <c r="F22">
+        <f t="shared" si="7"/>
+        <v>260452.77631578947</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="8"/>
+        <v>279938.14777407999</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B23">
+        <f t="shared" ref="B23:C23" si="13">B10*31.104</f>
+        <v>1664.4481753776663</v>
+      </c>
+      <c r="C23">
+        <f t="shared" si="13"/>
+        <v>2219.256740777917</v>
+      </c>
+      <c r="F23">
+        <f t="shared" si="7"/>
+        <v>278956.46511627908</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="8"/>
+        <v>148088</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B24">
+        <f t="shared" ref="B24:C24" si="14">B11*31.104</f>
+        <v>1664.4481753776663</v>
+      </c>
+      <c r="C24">
+        <f t="shared" si="14"/>
+        <v>277.40428270012541</v>
+      </c>
+      <c r="F24">
+        <f t="shared" si="7"/>
+        <v>333764.02249175153</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="8"/>
+        <v>148088.00000000003</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B25">
+        <f t="shared" ref="B25:C25" si="15">B12*31.104</f>
+        <v>1664.4481753776663</v>
+      </c>
+      <c r="C25">
+        <f t="shared" si="15"/>
+        <v>1387.0326530890841</v>
+      </c>
+      <c r="F25">
+        <f t="shared" si="7"/>
+        <v>471353.99516706169</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="8"/>
+        <v>148088.00000000003</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B26">
+        <f t="shared" ref="B26:C26" si="16">B13*31.104</f>
+        <v>1664.4481753776663</v>
+      </c>
+      <c r="C26">
+        <f t="shared" si="16"/>
+        <v>1109.6283703889585</v>
+      </c>
+      <c r="F26">
+        <f t="shared" si="7"/>
+        <v>155808.05255820439</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="8"/>
+        <v>148088.00000000003</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F27">
+        <f t="shared" si="7"/>
+        <v>279878.19870811841</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="8"/>
+        <v>148088.00000000003</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F28">
+        <f t="shared" si="7"/>
+        <v>235169.14805520704</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="8"/>
+        <v>148088.00000000003</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E31" t="s">
+        <v>12</v>
+      </c>
+      <c r="F31">
+        <f>SUM(F17:F28)</f>
+        <v>3879440.5531492536</v>
+      </c>
+      <c r="G31">
+        <f>SUM(G17:G28)</f>
+        <v>3420879.3241951307</v>
+      </c>
+      <c r="H31">
+        <f>100*(F31-G31)/F31</f>
+        <v>11.820292711583681</v>
+      </c>
+    </row>
+    <row r="32" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E32" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32">
+        <f>0.05*SUM(K2:K13)</f>
+        <v>0</v>
+      </c>
+      <c r="G32">
+        <v>162857.60000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
+      </c>
+      <c r="G33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E34" t="s">
+        <v>15</v>
+      </c>
+      <c r="F34">
+        <f>SUM(F31:F33)</f>
+        <v>3879440.5531492536</v>
+      </c>
+      <c r="G34">
+        <f>SUM(G31:G33)</f>
+        <v>3583736.9241951308</v>
+      </c>
+      <c r="H34">
+        <f t="shared" ref="H34" si="17">100*(F34-G34)/F34</f>
+        <v>7.6223265933041908</v>
+      </c>
+    </row>
+    <row r="36" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E36" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="37" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E37" t="s">
+        <v>12</v>
+      </c>
+      <c r="F37">
+        <v>3661</v>
+      </c>
+      <c r="G37">
+        <f>F37*(1-H31/100)</f>
+        <v>3228.2590838289216</v>
+      </c>
+      <c r="H37">
+        <f>F37-G37</f>
+        <v>432.74091617107842</v>
+      </c>
+    </row>
+    <row r="38" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E38" t="s">
+        <v>13</v>
+      </c>
+      <c r="F38">
+        <f>F32*F37/F31</f>
+        <v>0</v>
+      </c>
+      <c r="G38">
+        <f>F38*(1-H32/100)</f>
+        <v>0</v>
+      </c>
+      <c r="H38">
+        <f t="shared" ref="H38:H39" si="18">F38-G38</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E39" t="s">
+        <v>14</v>
+      </c>
+      <c r="F39">
+        <v>0</v>
+      </c>
+      <c r="G39">
+        <f>F39*(1-H33/100)</f>
+        <v>0</v>
+      </c>
+      <c r="H39">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E40" t="s">
+        <v>15</v>
+      </c>
+      <c r="F40">
+        <f>SUM(F37:F39)</f>
+        <v>3661</v>
+      </c>
+      <c r="G40">
+        <f>SUM(G37:G39)</f>
+        <v>3228.2590838289216</v>
+      </c>
+      <c r="H40">
+        <f>SUM(H37:H39)</f>
+        <v>432.74091617107842</v>
       </c>
     </row>
   </sheetData>
@@ -935,8 +1336,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34E3220C-D6E8-CA4D-AC53-28C815E97289}">
-  <dimension ref="A1:L13"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35D93EDA-C388-0E49-820D-284E95AE45F4}">
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="12.6640625" customWidth="1"/>
@@ -1004,22 +1405,21 @@
       <c r="G2" s="2">
         <v>4886.8312757201647</v>
       </c>
-      <c r="H2" s="4">
-        <v>7000</v>
+      <c r="H2">
+        <v>9513.1687242798362</v>
       </c>
       <c r="I2">
         <f>SUM(G2:H2)</f>
-        <v>11886.831275720164</v>
+        <v>14400</v>
       </c>
       <c r="J2" s="4">
         <v>10314.285714285714</v>
       </c>
       <c r="K2">
-        <f>F2-J2</f>
         <v>4085.7142857142862</v>
       </c>
       <c r="L2">
-        <v>2113.1687242798344</v>
+        <v>804.54556143445006</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
@@ -1046,21 +1446,21 @@
         <v>4886.8312757201647</v>
       </c>
       <c r="H3" s="4">
-        <v>7000</v>
+        <v>4000</v>
       </c>
       <c r="I3">
         <f t="shared" ref="I3:I13" si="1">SUM(G3:H3)</f>
-        <v>11886.831275720164</v>
+        <v>8886.8312757201638</v>
       </c>
       <c r="J3">
-        <v>5907.1382972953343</v>
+        <v>12000</v>
       </c>
       <c r="K3">
-        <f>K2+F3-J3</f>
         <v>3258.3084987070179</v>
       </c>
       <c r="L3">
-        <v>8920.2674897119323</v>
+        <f>L2+I3-J3</f>
+        <v>-2308.6231628453861</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
@@ -1087,21 +1487,21 @@
         <v>4886.8312757201647</v>
       </c>
       <c r="H4" s="4">
-        <v>7000</v>
+        <v>5000</v>
       </c>
       <c r="I4">
         <f t="shared" si="1"/>
-        <v>11886.831275720164</v>
+        <v>9886.8312757201638</v>
       </c>
       <c r="J4">
         <v>5625.7573205650187</v>
       </c>
       <c r="K4">
-        <f t="shared" ref="K4:K13" si="2">K3+F4-J4</f>
         <v>7534.8145526275966</v>
       </c>
       <c r="L4">
-        <v>10904.835390946499</v>
+        <f t="shared" ref="L4:L13" si="2">L3+I4-J4</f>
+        <v>1952.450792309759</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -1128,21 +1528,21 @@
         <v>4886.8312757201647</v>
       </c>
       <c r="H5" s="4">
-        <v>7000</v>
+        <v>2000</v>
       </c>
       <c r="I5">
         <f t="shared" si="1"/>
-        <v>11886.831275720164</v>
+        <v>6886.8312757201647</v>
       </c>
       <c r="J5">
         <v>6433.9826158977739</v>
       </c>
       <c r="K5">
+        <v>9427.7352289108931</v>
+      </c>
+      <c r="L5">
         <f t="shared" si="2"/>
-        <v>9427.7352289108931</v>
-      </c>
-      <c r="L5">
-        <v>14464.763374485594</v>
+        <v>2405.2994521321489</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
@@ -1169,21 +1569,21 @@
         <v>4886.8312757201647</v>
       </c>
       <c r="H6" s="4">
-        <v>6657.9218106995604</v>
+        <v>7000</v>
       </c>
       <c r="I6">
         <f t="shared" si="1"/>
-        <v>11544.753086419725</v>
+        <v>11886.831275720164</v>
       </c>
       <c r="J6">
         <v>6493.9081133646077</v>
       </c>
       <c r="K6">
+        <v>11260.730407727355</v>
+      </c>
+      <c r="L6">
         <f t="shared" si="2"/>
-        <v>11260.730407727355</v>
-      </c>
-      <c r="L6">
-        <v>17682.613168724245</v>
+        <v>7798.222614487705</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
@@ -1210,21 +1610,21 @@
         <v>4886.8312757201647</v>
       </c>
       <c r="H7" s="4">
-        <v>3279.3186831275698</v>
+        <v>7000</v>
       </c>
       <c r="I7">
         <f t="shared" si="1"/>
-        <v>8166.1499588477345</v>
+        <v>11886.831275720164</v>
       </c>
       <c r="J7">
-        <v>6071.2326312903115</v>
+        <v>8000</v>
       </c>
       <c r="K7">
+        <v>11426.637694132516</v>
+      </c>
+      <c r="L7">
         <f t="shared" si="2"/>
-        <v>11426.637694132516</v>
-      </c>
-      <c r="L7">
-        <v>19611.623209876507</v>
+        <v>11685.05389020787</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
@@ -1251,21 +1651,21 @@
         <v>2764.9176954732511</v>
       </c>
       <c r="H8" s="4">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="I8">
         <f t="shared" si="1"/>
-        <v>2764.9176954732511</v>
+        <v>12764.91769547325</v>
       </c>
       <c r="J8">
-        <v>6403.8158313631438</v>
+        <v>15000</v>
       </c>
       <c r="K8">
+        <v>10231.155196102707</v>
+      </c>
+      <c r="L8">
         <f t="shared" si="2"/>
-        <v>10231.155196102707</v>
-      </c>
-      <c r="L8">
-        <v>17168.207572016425</v>
+        <v>9449.9715856811199</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
@@ -1292,21 +1692,21 @@
         <v>2767.3611111111113</v>
       </c>
       <c r="H9" s="4">
-        <v>0</v>
+        <v>10500</v>
       </c>
       <c r="I9">
         <f t="shared" si="1"/>
-        <v>2767.3611111111113</v>
+        <v>13267.361111111111</v>
       </c>
       <c r="J9">
-        <v>6026.4848889003415</v>
+        <v>15000</v>
       </c>
       <c r="K9">
+        <v>10441.810224897839</v>
+      </c>
+      <c r="L9">
         <f t="shared" si="2"/>
-        <v>10441.810224897839</v>
-      </c>
-      <c r="L9">
-        <v>13698.428765432065</v>
+        <v>7717.332696792233</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
@@ -1333,21 +1733,21 @@
         <v>2767.3611111111113</v>
       </c>
       <c r="H10" s="4">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="I10">
         <f t="shared" si="1"/>
-        <v>2767.3611111111113</v>
+        <v>12767.361111111111</v>
       </c>
       <c r="J10">
-        <v>4479.7985738060161</v>
+        <v>9000</v>
       </c>
       <c r="K10">
+        <v>13260.108358910755</v>
+      </c>
+      <c r="L10">
         <f t="shared" si="2"/>
-        <v>13260.108358910755</v>
-      </c>
-      <c r="L10">
-        <v>9167.6931687242432</v>
+        <v>11484.693807903343</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
@@ -1381,14 +1781,14 @@
         <v>2767.3611111111113</v>
       </c>
       <c r="J11">
-        <v>4284.164832400751</v>
+        <v>7000</v>
       </c>
       <c r="K11">
+        <v>12608.916777538809</v>
+      </c>
+      <c r="L11">
         <f t="shared" si="2"/>
-        <v>12608.916777538809</v>
-      </c>
-      <c r="L11">
-        <v>8302.0810288065477</v>
+        <v>7252.0549190144538</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
@@ -1422,14 +1822,14 @@
         <v>2767.3611111111113</v>
       </c>
       <c r="J12">
-        <v>3874.8158713185621</v>
+        <v>7000</v>
       </c>
       <c r="K12">
+        <v>14456.837531734651</v>
+      </c>
+      <c r="L12">
         <f t="shared" si="2"/>
-        <v>14456.837531734651</v>
-      </c>
-      <c r="L12">
-        <v>5346.7055144032556</v>
+        <v>3019.4160301255652</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
@@ -1466,11 +1866,270 @@
         <v>3826.840185484803</v>
       </c>
       <c r="K13">
+        <v>15838.33067958318</v>
+      </c>
+      <c r="L13">
         <f t="shared" si="2"/>
-        <v>15838.33067958318</v>
-      </c>
-      <c r="L13">
-        <v>2905.7332921810339</v>
+        <v>1959.9369557518735</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="F16" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F17">
+        <f>B2*D2+C2*E2</f>
+        <v>20896.148657136669</v>
+      </c>
+      <c r="G17">
+        <f>B2*G2+C2*H2</f>
+        <v>20896.148657136669</v>
+      </c>
+    </row>
+    <row r="18" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F18">
+        <f t="shared" ref="F18:F28" si="3">B3*D3+C3*E3</f>
+        <v>7724.5691872427979</v>
+      </c>
+      <c r="G18">
+        <f t="shared" ref="G18:G28" si="4">B3*G3+C3*H3</f>
+        <v>7724.5691872427979</v>
+      </c>
+    </row>
+    <row r="19" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F19">
+        <f t="shared" si="3"/>
+        <v>15264.614806692658</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="4"/>
+        <v>15242.062418778427</v>
+      </c>
+    </row>
+    <row r="20" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F20">
+        <f t="shared" si="3"/>
+        <v>11286.624160710418</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="4"/>
+        <v>9883.6150503573754</v>
+      </c>
+    </row>
+    <row r="21" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F21">
+        <f t="shared" si="3"/>
+        <v>11286.624160710418</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="4"/>
+        <v>14754.93083983106</v>
+      </c>
+    </row>
+    <row r="22" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F22">
+        <f t="shared" si="3"/>
+        <v>8373.6103496588712</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="4"/>
+        <v>10208.38478719948</v>
+      </c>
+    </row>
+    <row r="23" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F23">
+        <f t="shared" si="3"/>
+        <v>8968.5077519379847</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="4"/>
+        <v>21980.594554502823</v>
+      </c>
+    </row>
+    <row r="24" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F24">
+        <f t="shared" si="3"/>
+        <v>10730.581998834603</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="4"/>
+        <v>22825.607279871532</v>
+      </c>
+    </row>
+    <row r="25" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F25">
+        <f t="shared" si="3"/>
+        <v>15154.127931039791</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="4"/>
+        <v>27700.090294881527</v>
+      </c>
+    </row>
+    <row r="26" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F26">
+        <f t="shared" si="3"/>
+        <v>5009.260949016345</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="4"/>
+        <v>4761.0596707818931</v>
+      </c>
+    </row>
+    <row r="27" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F27">
+        <f t="shared" si="3"/>
+        <v>8998.1416765727372</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="4"/>
+        <v>4761.0596707818931</v>
+      </c>
+    </row>
+    <row r="28" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F28">
+        <f t="shared" si="3"/>
+        <v>7560.7364986884968</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="4"/>
+        <v>4761.0596707818931</v>
+      </c>
+    </row>
+    <row r="31" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E31" t="s">
+        <v>12</v>
+      </c>
+      <c r="F31">
+        <f>SUM(F17:F28)</f>
+        <v>131253.54812824179</v>
+      </c>
+      <c r="G31">
+        <f>SUM(G17:G28)</f>
+        <v>165499.18208214737</v>
+      </c>
+      <c r="H31">
+        <f>100*(F31-G31)/F31</f>
+        <v>-26.091206251007971</v>
+      </c>
+    </row>
+    <row r="32" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E32" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32">
+        <f>0.05*SUM(K2:K13)</f>
+        <v>6191.5549718293805</v>
+      </c>
+      <c r="G32">
+        <f>0.05*SUM(L2:L13)</f>
+        <v>3161.0177571497566</v>
+      </c>
+      <c r="H32">
+        <f t="shared" ref="H32:H34" si="5">100*(F32-G32)/F32</f>
+        <v>48.946302317723095</v>
+      </c>
+    </row>
+    <row r="33" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
+      </c>
+      <c r="G33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E34" t="s">
+        <v>15</v>
+      </c>
+      <c r="F34">
+        <f>SUM(F31:F33)</f>
+        <v>137445.10310007117</v>
+      </c>
+      <c r="G34">
+        <f>SUM(G31:G33)</f>
+        <v>168660.19983929713</v>
+      </c>
+      <c r="H34">
+        <f t="shared" si="5"/>
+        <v>-22.710955890875827</v>
+      </c>
+    </row>
+    <row r="36" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E36" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="37" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E37" t="s">
+        <v>12</v>
+      </c>
+      <c r="F37">
+        <v>4064</v>
+      </c>
+      <c r="G37">
+        <v>3960.48</v>
+      </c>
+      <c r="H37">
+        <f>F37-G37</f>
+        <v>103.51999999999998</v>
+      </c>
+    </row>
+    <row r="38" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E38" t="s">
+        <v>13</v>
+      </c>
+      <c r="F38">
+        <v>191.7</v>
+      </c>
+      <c r="G38">
+        <f>F38+48.8</f>
+        <v>240.5</v>
+      </c>
+      <c r="H38">
+        <f t="shared" ref="H38:H39" si="6">F38-G38</f>
+        <v>-48.800000000000011</v>
+      </c>
+    </row>
+    <row r="39" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E39" t="s">
+        <v>14</v>
+      </c>
+      <c r="F39">
+        <v>0</v>
+      </c>
+      <c r="G39">
+        <f>F39*(1-H33/100)</f>
+        <v>0</v>
+      </c>
+      <c r="H39">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E40" t="s">
+        <v>15</v>
+      </c>
+      <c r="F40">
+        <f>SUM(F37:F39)</f>
+        <v>4255.7</v>
+      </c>
+      <c r="G40">
+        <f>SUM(G37:G39)</f>
+        <v>4200.9799999999996</v>
+      </c>
+      <c r="H40">
+        <f>SUM(H37:H39)</f>
+        <v>54.71999999999997</v>
       </c>
     </row>
   </sheetData>
@@ -1480,8 +2139,8 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A487B8A4-70A8-BF44-BD3B-04E3E6FA5695}">
-  <dimension ref="A1:L13"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34E3220C-D6E8-CA4D-AC53-28C815E97289}">
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="12.6640625" customWidth="1"/>
@@ -1550,11 +2209,11 @@
         <v>4886.8312757201647</v>
       </c>
       <c r="H2" s="4">
-        <v>7000</v>
+        <v>6232</v>
       </c>
       <c r="I2">
         <f>SUM(G2:H2)</f>
-        <v>11886.831275720164</v>
+        <v>11118.831275720164</v>
       </c>
       <c r="J2" s="4">
         <v>10314.285714285714</v>
@@ -1564,7 +2223,7 @@
         <v>4085.7142857142862</v>
       </c>
       <c r="L2">
-        <v>2113.1687242798344</v>
+        <v>804.54556143445006</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
@@ -1581,11 +2240,11 @@
         <v>4886.8312757201647</v>
       </c>
       <c r="E3" s="2">
-        <v>2570.3115814226921</v>
+        <v>192.90123456790116</v>
       </c>
       <c r="F3">
         <f t="shared" ref="F3:F13" si="0">SUM(D3:E3)</f>
-        <v>7457.1428571428569</v>
+        <v>5079.7325102880659</v>
       </c>
       <c r="G3" s="2">
         <v>4886.8312757201647</v>
@@ -1597,15 +2256,16 @@
         <f t="shared" ref="I3:I13" si="1">SUM(G3:H3)</f>
         <v>11886.831275720164</v>
       </c>
-      <c r="J3" s="4">
+      <c r="J3">
         <v>12000</v>
       </c>
       <c r="K3">
         <f>K2+F3-J3</f>
-        <v>-457.14285714285688</v>
+        <v>-2834.5532039976479</v>
       </c>
       <c r="L3">
-        <v>8920.2674897119323</v>
+        <f>L2+I3-J3</f>
+        <v>691.3768371546139</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
@@ -1632,21 +2292,22 @@
         <v>4886.8312757201647</v>
       </c>
       <c r="H4" s="4">
-        <v>7000</v>
+        <v>1000</v>
       </c>
       <c r="I4">
         <f t="shared" si="1"/>
-        <v>11886.831275720164</v>
+        <v>5886.8312757201647</v>
       </c>
       <c r="J4">
         <v>5625.7573205650187</v>
       </c>
       <c r="K4">
         <f t="shared" ref="K4:K13" si="2">K3+F4-J4</f>
-        <v>3819.3631967777219</v>
+        <v>1441.9528499229309</v>
       </c>
       <c r="L4">
-        <v>10904.835390946499</v>
+        <f t="shared" ref="L4:L13" si="3">L3+I4-J4</f>
+        <v>952.45079230975989</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -1684,10 +2345,11 @@
       </c>
       <c r="K5">
         <f t="shared" si="2"/>
-        <v>5712.2838730610183</v>
+        <v>3334.8735262062273</v>
       </c>
       <c r="L5">
-        <v>14464.763374485594</v>
+        <f t="shared" si="3"/>
+        <v>6405.2994521321489</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
@@ -1714,21 +2376,22 @@
         <v>4886.8312757201647</v>
       </c>
       <c r="H6" s="4">
-        <v>6657.9218106995604</v>
+        <v>4500</v>
       </c>
       <c r="I6">
         <f t="shared" si="1"/>
-        <v>11544.753086419725</v>
+        <v>9386.8312757201638</v>
       </c>
       <c r="J6">
         <v>6493.9081133646077</v>
       </c>
       <c r="K6">
         <f t="shared" si="2"/>
-        <v>7545.2790518774809</v>
+        <v>5167.8687050226899</v>
       </c>
       <c r="L6">
-        <v>17682.613168724245</v>
+        <f t="shared" si="3"/>
+        <v>9298.2226144877059</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
@@ -1755,21 +2418,22 @@
         <v>4886.8312757201647</v>
       </c>
       <c r="H7" s="4">
-        <v>3279.3186831275698</v>
+        <v>3000</v>
       </c>
       <c r="I7">
         <f t="shared" si="1"/>
-        <v>8166.1499588477345</v>
+        <v>7886.8312757201647</v>
       </c>
       <c r="J7">
         <v>6071.2326312903115</v>
       </c>
       <c r="K7">
         <f t="shared" si="2"/>
-        <v>7711.1863382826432</v>
+        <v>5333.7759914278522</v>
       </c>
       <c r="L7">
-        <v>19611.623209876507</v>
+        <f t="shared" si="3"/>
+        <v>11113.821258917558</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
@@ -1796,21 +2460,22 @@
         <v>2764.9176954732511</v>
       </c>
       <c r="H8" s="4">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="I8">
         <f t="shared" si="1"/>
-        <v>2764.9176954732511</v>
+        <v>7764.9176954732511</v>
       </c>
       <c r="J8">
         <v>6403.8158313631438</v>
       </c>
       <c r="K8">
         <f t="shared" si="2"/>
-        <v>6515.7038402528333</v>
+        <v>4138.2934933980423</v>
       </c>
       <c r="L8">
-        <v>17168.207572016425</v>
+        <f t="shared" si="3"/>
+        <v>12474.923123027667</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
@@ -1837,21 +2502,22 @@
         <v>2767.3611111111113</v>
       </c>
       <c r="H9" s="4">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="I9">
         <f t="shared" si="1"/>
-        <v>2767.3611111111113</v>
+        <v>7767.3611111111113</v>
       </c>
       <c r="J9">
         <v>6026.4848889003415</v>
       </c>
       <c r="K9">
         <f t="shared" si="2"/>
-        <v>6726.3588690479655</v>
+        <v>4348.9485221931745</v>
       </c>
       <c r="L9">
-        <v>13698.428765432065</v>
+        <f t="shared" si="3"/>
+        <v>14215.79934523844</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
@@ -1878,21 +2544,22 @@
         <v>2767.3611111111113</v>
       </c>
       <c r="H10" s="4">
-        <v>0</v>
+        <v>2300</v>
       </c>
       <c r="I10">
         <f t="shared" si="1"/>
-        <v>2767.3611111111113</v>
+        <v>5067.3611111111113</v>
       </c>
       <c r="J10">
-        <v>4479.7985738060161</v>
+        <v>7000</v>
       </c>
       <c r="K10">
         <f t="shared" si="2"/>
-        <v>9544.65700306088</v>
+        <v>4647.0452300121051</v>
       </c>
       <c r="L10">
-        <v>9167.6931687242432</v>
+        <f t="shared" si="3"/>
+        <v>12283.160456349549</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
@@ -1919,21 +2586,22 @@
         <v>2767.3611111111113</v>
       </c>
       <c r="H11" s="4">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="I11">
         <f t="shared" si="1"/>
-        <v>2767.3611111111113</v>
+        <v>5267.3611111111113</v>
       </c>
       <c r="J11">
         <v>4284.164832400751</v>
       </c>
       <c r="K11">
         <f t="shared" si="2"/>
-        <v>8893.4654216889357</v>
+        <v>3995.8536486401608</v>
       </c>
       <c r="L11">
-        <v>8302.0810288065477</v>
+        <f t="shared" si="3"/>
+        <v>13266.356735059908</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
@@ -1971,10 +2639,11 @@
       </c>
       <c r="K12">
         <f t="shared" si="2"/>
-        <v>10741.386175884778</v>
+        <v>5843.774402836003</v>
       </c>
       <c r="L12">
-        <v>5346.7055144032556</v>
+        <f t="shared" si="3"/>
+        <v>12158.901974852457</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
@@ -2012,10 +2681,270 @@
       </c>
       <c r="K13">
         <f t="shared" si="2"/>
-        <v>12122.879323733307</v>
+        <v>7225.2675506845317</v>
       </c>
       <c r="L13">
-        <v>2905.7332921810339</v>
+        <f t="shared" si="3"/>
+        <v>11099.422900478765</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="F16" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F17">
+        <f>B2*D2+C2*E2</f>
+        <v>20896.148657136669</v>
+      </c>
+      <c r="G17">
+        <f>B2*G2+C2*H2</f>
+        <v>16265.728814814815</v>
+      </c>
+    </row>
+    <row r="18" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F18">
+        <f t="shared" ref="F18:F28" si="4">B3*D3+C3*E3</f>
+        <v>7724.5691872427979</v>
+      </c>
+      <c r="G18">
+        <f t="shared" ref="G18:G28" si="5">B3*G3+C3*H3</f>
+        <v>7724.5691872427979</v>
+      </c>
+    </row>
+    <row r="19" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F19">
+        <f t="shared" si="4"/>
+        <v>15264.614806692658</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="5"/>
+        <v>9396.483471410007</v>
+      </c>
+    </row>
+    <row r="20" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F20">
+        <f t="shared" si="4"/>
+        <v>11286.624160710418</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="5"/>
+        <v>14754.93083983106</v>
+      </c>
+    </row>
+    <row r="21" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F21">
+        <f t="shared" si="4"/>
+        <v>11286.624160710418</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="5"/>
+        <v>12319.272945094217</v>
+      </c>
+    </row>
+    <row r="22" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F22">
+        <f t="shared" si="4"/>
+        <v>8373.6103496588712</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="5"/>
+        <v>8909.358471410007</v>
+      </c>
+    </row>
+    <row r="23" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F23">
+        <f t="shared" si="4"/>
+        <v>8968.5077519379847</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="5"/>
+        <v>13370.827112642359</v>
+      </c>
+    </row>
+    <row r="24" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F24">
+        <f t="shared" si="4"/>
+        <v>10730.581998834603</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="5"/>
+        <v>13363.225198919818</v>
+      </c>
+    </row>
+    <row r="25" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F25">
+        <f t="shared" si="4"/>
+        <v>15154.127931039791</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="5"/>
+        <v>10037.036714324808</v>
+      </c>
+    </row>
+    <row r="26" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F26">
+        <f t="shared" si="4"/>
+        <v>5009.260949016345</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="5"/>
+        <v>5477.8971167598665</v>
+      </c>
+    </row>
+    <row r="27" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F27">
+        <f t="shared" si="4"/>
+        <v>8998.1416765727372</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="5"/>
+        <v>4761.0596707818931</v>
+      </c>
+    </row>
+    <row r="28" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F28">
+        <f t="shared" si="4"/>
+        <v>7560.7364986884968</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="5"/>
+        <v>4761.0596707818931</v>
+      </c>
+    </row>
+    <row r="31" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E31" t="s">
+        <v>12</v>
+      </c>
+      <c r="F31">
+        <f>SUM(F17:F28)</f>
+        <v>131253.54812824179</v>
+      </c>
+      <c r="G31">
+        <f>SUM(G17:G28)</f>
+        <v>121141.44921401354</v>
+      </c>
+      <c r="H31">
+        <f>100*(F31-G31)/F31</f>
+        <v>7.7042480439067322</v>
+      </c>
+    </row>
+    <row r="32" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E32" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32">
+        <f>0.05*SUM(K2:K13)</f>
+        <v>2336.4407501030178</v>
+      </c>
+      <c r="G32">
+        <f>0.05*SUM(L2:L13)</f>
+        <v>5238.2140525721516</v>
+      </c>
+      <c r="H32">
+        <f t="shared" ref="H32:H34" si="6">100*(F32-G32)/F32</f>
+        <v>-124.19631451562336</v>
+      </c>
+    </row>
+    <row r="33" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
+      </c>
+      <c r="G33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E34" t="s">
+        <v>15</v>
+      </c>
+      <c r="F34">
+        <f>SUM(F31:F33)</f>
+        <v>133589.9888783448</v>
+      </c>
+      <c r="G34">
+        <f>SUM(G31:G33)</f>
+        <v>126379.66326658569</v>
+      </c>
+      <c r="H34">
+        <f t="shared" si="6"/>
+        <v>5.3973547511297948</v>
+      </c>
+    </row>
+    <row r="36" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E36" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="37" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E37" t="s">
+        <v>12</v>
+      </c>
+      <c r="F37">
+        <v>4064</v>
+      </c>
+      <c r="G37">
+        <v>3960.48</v>
+      </c>
+      <c r="H37">
+        <f>F37-G37</f>
+        <v>103.51999999999998</v>
+      </c>
+    </row>
+    <row r="38" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E38" t="s">
+        <v>13</v>
+      </c>
+      <c r="F38">
+        <v>191.7</v>
+      </c>
+      <c r="G38">
+        <f>F38+48.8</f>
+        <v>240.5</v>
+      </c>
+      <c r="H38">
+        <f t="shared" ref="H38:H39" si="7">F38-G38</f>
+        <v>-48.800000000000011</v>
+      </c>
+    </row>
+    <row r="39" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E39" t="s">
+        <v>14</v>
+      </c>
+      <c r="F39">
+        <v>0</v>
+      </c>
+      <c r="G39">
+        <f>F39*(1-H33/100)</f>
+        <v>0</v>
+      </c>
+      <c r="H39">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E40" t="s">
+        <v>15</v>
+      </c>
+      <c r="F40">
+        <f>SUM(F37:F39)</f>
+        <v>4255.7</v>
+      </c>
+      <c r="G40">
+        <f>SUM(G37:G39)</f>
+        <v>4200.9799999999996</v>
+      </c>
+      <c r="H40">
+        <f>SUM(H37:H39)</f>
+        <v>54.71999999999997</v>
       </c>
     </row>
   </sheetData>
@@ -2025,8 +2954,827 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A487B8A4-70A8-BF44-BD3B-04E3E6FA5695}">
+  <dimension ref="A1:L40"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="15.6640625" customWidth="1"/>
+    <col min="6" max="6" width="12.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="41" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
+        <v>45772</v>
+      </c>
+      <c r="B2">
+        <v>1.5288157894736842</v>
+      </c>
+      <c r="C2">
+        <v>1.4112105263157895</v>
+      </c>
+      <c r="D2" s="2">
+        <v>4886.8312757201647</v>
+      </c>
+      <c r="E2" s="2">
+        <v>9513.1687242798362</v>
+      </c>
+      <c r="F2">
+        <f>SUM(D2:E2)</f>
+        <v>14400</v>
+      </c>
+      <c r="G2" s="2">
+        <v>4886.8312757201647</v>
+      </c>
+      <c r="H2">
+        <v>9513.1687242798362</v>
+      </c>
+      <c r="I2">
+        <f>SUM(G2:H2)</f>
+        <v>14400</v>
+      </c>
+      <c r="J2" s="4">
+        <v>10314.285714285714</v>
+      </c>
+      <c r="K2">
+        <f>F2-J2</f>
+        <v>4085.7142857142862</v>
+      </c>
+      <c r="L2">
+        <f>1000+I2-J2</f>
+        <v>5085.7142857142862</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>45802</v>
+      </c>
+      <c r="B3">
+        <v>1.5806907894736841</v>
+      </c>
+      <c r="C3">
+        <v>1.4112105263157895</v>
+      </c>
+      <c r="D3" s="2">
+        <v>4886.8312757201647</v>
+      </c>
+      <c r="E3" s="2">
+        <v>2570.3115814226921</v>
+      </c>
+      <c r="F3">
+        <f t="shared" ref="F3:F13" si="0">SUM(D3:E3)</f>
+        <v>7457.1428571428569</v>
+      </c>
+      <c r="G3" s="2">
+        <v>4886.8312757201647</v>
+      </c>
+      <c r="H3">
+        <v>2570.3115814226921</v>
+      </c>
+      <c r="I3">
+        <f t="shared" ref="I3:I13" si="1">SUM(G3:H3)</f>
+        <v>7457.1428571428569</v>
+      </c>
+      <c r="J3" s="4">
+        <v>12000</v>
+      </c>
+      <c r="K3">
+        <f>K2+F3-J3+1500</f>
+        <v>1042.8571428571431</v>
+      </c>
+      <c r="L3">
+        <f>L2+I3-J3</f>
+        <v>542.85714285714312</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
+        <v>45833</v>
+      </c>
+      <c r="B4">
+        <v>1.6237697368421053</v>
+      </c>
+      <c r="C4">
+        <v>1.4613947368421052</v>
+      </c>
+      <c r="D4" s="2">
+        <v>4886.8312757201647</v>
+      </c>
+      <c r="E4" s="2">
+        <v>5015.4320987654328</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="0"/>
+        <v>9902.2633744855975</v>
+      </c>
+      <c r="G4" s="2">
+        <v>4886.8312757201647</v>
+      </c>
+      <c r="H4" s="4">
+        <v>7000</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="1"/>
+        <v>11886.831275720164</v>
+      </c>
+      <c r="J4">
+        <v>9828.5714285714294</v>
+      </c>
+      <c r="K4">
+        <f t="shared" ref="K4:K13" si="2">K3+F4-J4</f>
+        <v>1116.5490887713113</v>
+      </c>
+      <c r="L4">
+        <f t="shared" ref="L4:L13" si="3">L3+I4-J4</f>
+        <v>2601.1169900058776</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>45863</v>
+      </c>
+      <c r="B5">
+        <v>1.6237697368421053</v>
+      </c>
+      <c r="C5">
+        <v>0.97426315789473683</v>
+      </c>
+      <c r="D5" s="2">
+        <v>4886.8312757201647</v>
+      </c>
+      <c r="E5" s="2">
+        <v>3440.0720164609056</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="0"/>
+        <v>8326.9032921810704</v>
+      </c>
+      <c r="G5" s="2">
+        <v>4886.8312757201647</v>
+      </c>
+      <c r="H5" s="4">
+        <v>3000</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="1"/>
+        <v>7886.8312757201647</v>
+      </c>
+      <c r="J5">
+        <v>6433.9826158977739</v>
+      </c>
+      <c r="K5">
+        <f t="shared" si="2"/>
+        <v>3009.4697650546077</v>
+      </c>
+      <c r="L5">
+        <f t="shared" si="3"/>
+        <v>4053.9656498282675</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>45894</v>
+      </c>
+      <c r="B6">
+        <v>1.6237697368421053</v>
+      </c>
+      <c r="C6">
+        <v>0.97426315789473683</v>
+      </c>
+      <c r="D6" s="2">
+        <v>4886.8312757201647</v>
+      </c>
+      <c r="E6" s="2">
+        <v>3440.0720164609056</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="0"/>
+        <v>8326.9032921810704</v>
+      </c>
+      <c r="G6" s="2">
+        <v>4886.8312757201647</v>
+      </c>
+      <c r="H6" s="4">
+        <v>7000</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="1"/>
+        <v>11886.831275720164</v>
+      </c>
+      <c r="J6">
+        <v>6493.9081133646077</v>
+      </c>
+      <c r="K6">
+        <f t="shared" si="2"/>
+        <v>4842.4649438710703</v>
+      </c>
+      <c r="L6">
+        <f t="shared" si="3"/>
+        <v>9446.8888121838245</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>45925</v>
+      </c>
+      <c r="B7">
+        <v>1.6237697368421053</v>
+      </c>
+      <c r="C7">
+        <v>0.32475657894736842</v>
+      </c>
+      <c r="D7" s="2">
+        <v>4886.8312757201647</v>
+      </c>
+      <c r="E7" s="2">
+        <v>1350.308641975309</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>6237.1399176954737</v>
+      </c>
+      <c r="G7" s="2">
+        <v>4886.8312757201647</v>
+      </c>
+      <c r="H7" s="4">
+        <v>1279.31868312757</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="1"/>
+        <v>6166.1499588477345</v>
+      </c>
+      <c r="J7">
+        <v>6071.2326312903115</v>
+      </c>
+      <c r="K7">
+        <f t="shared" si="2"/>
+        <v>5008.3722302762326</v>
+      </c>
+      <c r="L7">
+        <f t="shared" si="3"/>
+        <v>9541.8061397412475</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
+        <v>45955</v>
+      </c>
+      <c r="B8">
+        <v>1.7219534883720931</v>
+      </c>
+      <c r="C8">
+        <v>1.7219534883720931</v>
+      </c>
+      <c r="D8" s="2">
+        <v>2764.9176954732511</v>
+      </c>
+      <c r="E8" s="2">
+        <v>2443.4156378600819</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="0"/>
+        <v>5208.333333333333</v>
+      </c>
+      <c r="G8" s="2">
+        <v>2764.9176954732511</v>
+      </c>
+      <c r="H8" s="4">
+        <v>3000</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="1"/>
+        <v>5764.9176954732511</v>
+      </c>
+      <c r="J8">
+        <v>6403.8158313631438</v>
+      </c>
+      <c r="K8">
+        <f t="shared" si="2"/>
+        <v>3812.8897322464209</v>
+      </c>
+      <c r="L8">
+        <f t="shared" si="3"/>
+        <v>8902.9080038513566</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>45986</v>
+      </c>
+      <c r="B9">
+        <v>1.720433105627585</v>
+      </c>
+      <c r="C9">
+        <v>1.720433105627585</v>
+      </c>
+      <c r="D9" s="2">
+        <v>2767.3611111111113</v>
+      </c>
+      <c r="E9" s="2">
+        <v>3469.7788065843624</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="0"/>
+        <v>6237.1399176954737</v>
+      </c>
+      <c r="G9" s="2">
+        <v>2767.3611111111113</v>
+      </c>
+      <c r="H9" s="4">
+        <v>2000</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="1"/>
+        <v>4767.3611111111113</v>
+      </c>
+      <c r="J9">
+        <v>6026.4848889003415</v>
+      </c>
+      <c r="K9">
+        <f t="shared" si="2"/>
+        <v>4023.5447610415531</v>
+      </c>
+      <c r="L9">
+        <f t="shared" si="3"/>
+        <v>7643.7842260621264</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
+        <v>46016</v>
+      </c>
+      <c r="B10">
+        <v>1.720433105627585</v>
+      </c>
+      <c r="C10">
+        <v>2.2939030624099632</v>
+      </c>
+      <c r="D10" s="2">
+        <v>2767.3611111111113</v>
+      </c>
+      <c r="E10" s="2">
+        <v>4530.7355967078192</v>
+      </c>
+      <c r="F10">
+        <f t="shared" si="0"/>
+        <v>7298.0967078189306</v>
+      </c>
+      <c r="G10" s="2">
+        <v>2767.3611111111113</v>
+      </c>
+      <c r="H10" s="4">
+        <v>2500</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="1"/>
+        <v>5267.3611111111113</v>
+      </c>
+      <c r="J10">
+        <v>4479.7985738060161</v>
+      </c>
+      <c r="K10">
+        <f t="shared" si="2"/>
+        <v>6841.8428950544676</v>
+      </c>
+      <c r="L10">
+        <f t="shared" si="3"/>
+        <v>8431.3467633672226</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
+        <v>46047</v>
+      </c>
+      <c r="B11">
+        <v>1.720433105627585</v>
+      </c>
+      <c r="C11">
+        <v>0.28673497839118917</v>
+      </c>
+      <c r="D11" s="2">
+        <v>2767.3611111111113</v>
+      </c>
+      <c r="E11" s="2">
+        <v>865.61213991769546</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="0"/>
+        <v>3632.9732510288068</v>
+      </c>
+      <c r="G11" s="2">
+        <v>2767.3611111111113</v>
+      </c>
+      <c r="H11" s="4">
+        <v>2343</v>
+      </c>
+      <c r="I11">
+        <f t="shared" si="1"/>
+        <v>5110.3611111111113</v>
+      </c>
+      <c r="J11">
+        <v>4284.164832400751</v>
+      </c>
+      <c r="K11">
+        <f t="shared" si="2"/>
+        <v>6190.6513136825233</v>
+      </c>
+      <c r="L11">
+        <f t="shared" si="3"/>
+        <v>9257.5430420775829</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
+        <v>46078</v>
+      </c>
+      <c r="B12">
+        <v>1.720433105627585</v>
+      </c>
+      <c r="C12">
+        <v>1.4336865095961708</v>
+      </c>
+      <c r="D12" s="2">
+        <v>2767.3611111111113</v>
+      </c>
+      <c r="E12" s="2">
+        <v>2955.3755144032921</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="0"/>
+        <v>5722.7366255144034</v>
+      </c>
+      <c r="G12" s="2">
+        <v>2767.3611111111113</v>
+      </c>
+      <c r="H12" s="4">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <f t="shared" si="1"/>
+        <v>2767.3611111111113</v>
+      </c>
+      <c r="J12">
+        <v>3874.8158713185621</v>
+      </c>
+      <c r="K12">
+        <f t="shared" si="2"/>
+        <v>8038.5720678783655</v>
+      </c>
+      <c r="L12">
+        <f t="shared" si="3"/>
+        <v>8150.0882818701321</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
+        <v>46106</v>
+      </c>
+      <c r="B13">
+        <v>1.720433105627585</v>
+      </c>
+      <c r="C13">
+        <v>1.1469515312049816</v>
+      </c>
+      <c r="D13" s="2">
+        <v>2767.3611111111113</v>
+      </c>
+      <c r="E13" s="2">
+        <v>2440.9722222222217</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="0"/>
+        <v>5208.333333333333</v>
+      </c>
+      <c r="G13" s="2">
+        <v>2767.3611111111113</v>
+      </c>
+      <c r="H13" s="4">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="1"/>
+        <v>2767.3611111111113</v>
+      </c>
+      <c r="J13">
+        <v>3826.840185484803</v>
+      </c>
+      <c r="K13">
+        <f t="shared" si="2"/>
+        <v>9420.0652157268942</v>
+      </c>
+      <c r="L13">
+        <f t="shared" si="3"/>
+        <v>7090.6092074964399</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="F16" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F17">
+        <f>B2*D2+C2*E2</f>
+        <v>20896.148657136669</v>
+      </c>
+      <c r="G17">
+        <f>B2*G2+C2*H2</f>
+        <v>20896.148657136669</v>
+      </c>
+    </row>
+    <row r="18" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F18">
+        <f t="shared" ref="F18:F28" si="4">B3*D3+C3*E3</f>
+        <v>11351.819946857884</v>
+      </c>
+      <c r="G18">
+        <f t="shared" ref="G18:G28" si="5">B3*G3+C3*H3</f>
+        <v>11351.819946857884</v>
+      </c>
+    </row>
+    <row r="19" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F19">
+        <f t="shared" si="4"/>
+        <v>15264.614806692658</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="5"/>
+        <v>18164.851892462641</v>
+      </c>
+    </row>
+    <row r="20" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F20">
+        <f t="shared" si="4"/>
+        <v>11286.624160710418</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="5"/>
+        <v>10857.878208252112</v>
+      </c>
+    </row>
+    <row r="21" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F21">
+        <f t="shared" si="4"/>
+        <v>11286.624160710418</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="5"/>
+        <v>14754.93083983106</v>
+      </c>
+    </row>
+    <row r="22" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F22">
+        <f t="shared" si="4"/>
+        <v>8373.6103496588712</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="5"/>
+        <v>8350.5558934838646</v>
+      </c>
+    </row>
+    <row r="23" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F23">
+        <f t="shared" si="4"/>
+        <v>8968.5077519379847</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="5"/>
+        <v>9926.9201358981736</v>
+      </c>
+    </row>
+    <row r="24" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F24">
+        <f t="shared" si="4"/>
+        <v>10730.581998834603</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="5"/>
+        <v>8201.9258820370633</v>
+      </c>
+    </row>
+    <row r="25" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F25">
+        <f t="shared" si="4"/>
+        <v>15154.127931039791</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="5"/>
+        <v>10495.817326806802</v>
+      </c>
+    </row>
+    <row r="26" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F26">
+        <f t="shared" si="4"/>
+        <v>5009.260949016345</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="5"/>
+        <v>5432.8797251524493</v>
+      </c>
+    </row>
+    <row r="27" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F27">
+        <f t="shared" si="4"/>
+        <v>8998.1416765727372</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="5"/>
+        <v>4761.0596707818931</v>
+      </c>
+    </row>
+    <row r="28" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F28">
+        <f t="shared" si="4"/>
+        <v>7560.7364986884968</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="5"/>
+        <v>4761.0596707818931</v>
+      </c>
+    </row>
+    <row r="31" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E31" t="s">
+        <v>12</v>
+      </c>
+      <c r="F31">
+        <f>SUM(F17:F28)</f>
+        <v>134880.79888785689</v>
+      </c>
+      <c r="G31">
+        <f>SUM(G17:G28)</f>
+        <v>127955.8478494825</v>
+      </c>
+      <c r="H31">
+        <f>100*(F31-G31)/F31</f>
+        <v>5.1341266477313505</v>
+      </c>
+    </row>
+    <row r="32" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E32" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32">
+        <f>0.05*SUM(K2:K13)</f>
+        <v>2871.6496721087442</v>
+      </c>
+      <c r="G32">
+        <f>0.05*SUM(L2:L13)</f>
+        <v>4037.4314272527754</v>
+      </c>
+      <c r="H32">
+        <f t="shared" ref="H32:H34" si="6">100*(F32-G32)/F32</f>
+        <v>-40.596238687010882</v>
+      </c>
+    </row>
+    <row r="33" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
+      </c>
+      <c r="G33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E34" t="s">
+        <v>15</v>
+      </c>
+      <c r="F34">
+        <f>SUM(F31:F33)</f>
+        <v>137752.44855996562</v>
+      </c>
+      <c r="G34">
+        <f>SUM(G31:G33)</f>
+        <v>131993.27927673527</v>
+      </c>
+      <c r="H34">
+        <f t="shared" si="6"/>
+        <v>4.1808108265482504</v>
+      </c>
+    </row>
+    <row r="36" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E36" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="37" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E37" t="s">
+        <v>12</v>
+      </c>
+      <c r="F37">
+        <v>3661</v>
+      </c>
+      <c r="G37">
+        <f>F37*(1-H31/100)</f>
+        <v>3473.0396234265554</v>
+      </c>
+      <c r="H37">
+        <f>F37-G37</f>
+        <v>187.96037657344459</v>
+      </c>
+    </row>
+    <row r="38" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E38" t="s">
+        <v>13</v>
+      </c>
+      <c r="F38">
+        <f>F32*F37/F31</f>
+        <v>77.943706860240084</v>
+      </c>
+      <c r="G38">
+        <f>F38*(1-H32/100)</f>
+        <v>109.58592013872722</v>
+      </c>
+      <c r="H38">
+        <f t="shared" ref="H38:H39" si="7">F38-G38</f>
+        <v>-31.642213278487134</v>
+      </c>
+    </row>
+    <row r="39" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E39" t="s">
+        <v>14</v>
+      </c>
+      <c r="F39">
+        <v>0</v>
+      </c>
+      <c r="G39">
+        <f>F39*(1-H33/100)</f>
+        <v>0</v>
+      </c>
+      <c r="H39">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E40" t="s">
+        <v>15</v>
+      </c>
+      <c r="F40">
+        <f>SUM(F37:F39)</f>
+        <v>3738.9437068602401</v>
+      </c>
+      <c r="G40">
+        <f>SUM(G37:G39)</f>
+        <v>3582.6255435652824</v>
+      </c>
+      <c r="H40">
+        <f>SUM(H37:H39)</f>
+        <v>156.31816329495746</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7E44A41-3F86-B94E-AB4B-AA39DD02AB15}">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="12.6640625" customWidth="1"/>
@@ -2084,32 +3832,31 @@
       <c r="D2" s="2">
         <v>4886.8312757201647</v>
       </c>
-      <c r="E2" s="2">
-        <v>9513.1687242798362</v>
+      <c r="E2" s="5">
+        <v>2483.1669423159556</v>
       </c>
       <c r="F2">
         <f>SUM(D2:E2)</f>
-        <v>14400</v>
+        <v>7369.9982180361203</v>
       </c>
       <c r="G2" s="2">
         <v>4886.8312757201647</v>
       </c>
-      <c r="H2" s="4">
-        <v>7000</v>
+      <c r="H2">
+        <v>9513.1687242798362</v>
       </c>
       <c r="I2">
         <f>SUM(G2:H2)</f>
-        <v>11886.831275720164</v>
-      </c>
-      <c r="J2" s="4">
-        <v>10314.285714285714</v>
+        <v>14400</v>
+      </c>
+      <c r="J2">
+        <v>5195.1035206425595</v>
       </c>
       <c r="K2">
-        <f>F2-J2</f>
-        <v>4085.7142857142862</v>
+        <v>4271.1183717419499</v>
       </c>
       <c r="L2">
-        <v>2113.1687242798344</v>
+        <v>4271.1183717419508</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
@@ -2125,32 +3872,31 @@
       <c r="D3" s="2">
         <v>4886.8312757201647</v>
       </c>
-      <c r="E3" s="2">
-        <v>2570.3115814226921</v>
+      <c r="E3" s="5">
+        <v>0</v>
       </c>
       <c r="F3">
         <f t="shared" ref="F3:F13" si="0">SUM(D3:E3)</f>
-        <v>7457.1428571428569</v>
+        <v>4886.8312757201647</v>
       </c>
       <c r="G3" s="2">
         <v>4886.8312757201647</v>
       </c>
-      <c r="H3" s="4">
-        <v>7000</v>
+      <c r="H3">
+        <v>2570.3115814226921</v>
       </c>
       <c r="I3">
         <f t="shared" ref="I3:I13" si="1">SUM(G3:H3)</f>
-        <v>11886.831275720164</v>
-      </c>
-      <c r="J3" s="4">
-        <v>12000</v>
+        <v>7457.1428571428569</v>
+      </c>
+      <c r="J3">
+        <v>5907.1382972953343</v>
       </c>
       <c r="K3">
-        <f>K2+F3-J3</f>
-        <v>-457.14285714285688</v>
+        <v>1654.4669661241915</v>
       </c>
       <c r="L3">
-        <v>8920.2674897119323</v>
+        <v>1654.4669661241915</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
@@ -2166,32 +3912,31 @@
       <c r="D4" s="2">
         <v>4886.8312757201647</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="5">
+        <v>2545.222790928924</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="0"/>
+        <v>7432.0540666490888</v>
+      </c>
+      <c r="G4" s="2">
+        <v>4886.8312757201647</v>
+      </c>
+      <c r="H4">
         <v>9627.4544385655499</v>
       </c>
-      <c r="F4">
-        <f t="shared" si="0"/>
+      <c r="I4">
+        <f t="shared" si="1"/>
         <v>14514.285714285714</v>
       </c>
-      <c r="G4" s="2">
-        <v>4886.8312757201647</v>
-      </c>
-      <c r="H4" s="4">
-        <v>7000</v>
-      </c>
-      <c r="I4">
-        <f t="shared" si="1"/>
-        <v>11886.831275720164</v>
-      </c>
-      <c r="J4" s="4">
-        <v>9828.5714285714294</v>
+      <c r="J4">
+        <v>5625.7573205650187</v>
       </c>
       <c r="K4">
-        <f t="shared" ref="K4:K13" si="2">K3+F4-J4</f>
-        <v>4228.5714285714275</v>
+        <v>3912.337898729279</v>
       </c>
       <c r="L4">
-        <v>10904.835390946499</v>
+        <v>3912.337898729279</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -2207,32 +3952,32 @@
       <c r="D5" s="2">
         <v>4886.8312757201647</v>
       </c>
-      <c r="E5" s="2">
-        <v>3440.0720164609056</v>
+      <c r="E5" s="5">
+        <v>1371.7405698790662</v>
       </c>
       <c r="F5">
         <f t="shared" si="0"/>
-        <v>8326.9032921810704</v>
+        <v>6258.571845599231</v>
       </c>
       <c r="G5" s="2">
         <v>4886.8312757201647</v>
       </c>
       <c r="H5" s="4">
-        <v>7000</v>
+        <v>4000</v>
       </c>
       <c r="I5">
         <f t="shared" si="1"/>
-        <v>11886.831275720164</v>
+        <v>8886.8312757201638</v>
       </c>
       <c r="J5">
         <v>6433.9826158977739</v>
       </c>
       <c r="K5">
-        <f t="shared" si="2"/>
-        <v>6121.4921048547239</v>
+        <v>3693.0744358561019</v>
       </c>
       <c r="L5">
-        <v>14464.763374485594</v>
+        <f>L4+I5-J5</f>
+        <v>6365.186558551668</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
@@ -2248,12 +3993,12 @@
       <c r="D6" s="2">
         <v>4886.8312757201647</v>
       </c>
-      <c r="E6" s="2">
-        <v>3440.0720164609056</v>
+      <c r="E6" s="5">
+        <v>1371.7405698790662</v>
       </c>
       <c r="F6">
         <f t="shared" si="0"/>
-        <v>8326.9032921810704</v>
+        <v>6258.571845599231</v>
       </c>
       <c r="G6" s="2">
         <v>4886.8312757201647</v>
@@ -2269,11 +4014,11 @@
         <v>6493.9081133646077</v>
       </c>
       <c r="K6">
-        <f t="shared" si="2"/>
-        <v>7954.4872836711866</v>
+        <v>3398.9041011493814</v>
       </c>
       <c r="L6">
-        <v>17682.613168724245</v>
+        <f t="shared" ref="L6:L13" si="2">L5+I6-J6</f>
+        <v>11416.031531606786</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
@@ -2289,32 +4034,32 @@
       <c r="D7" s="2">
         <v>4886.8312757201647</v>
       </c>
-      <c r="E7" s="2">
-        <v>1350.308641975309</v>
+      <c r="E7" s="5">
+        <v>0</v>
       </c>
       <c r="F7">
         <f t="shared" si="0"/>
-        <v>6237.1399176954737</v>
+        <v>4886.8312757201647</v>
       </c>
       <c r="G7" s="2">
         <v>4886.8312757201647</v>
       </c>
-      <c r="H7" s="4">
-        <v>3279.3186831275698</v>
+      <c r="H7">
+        <v>3000</v>
       </c>
       <c r="I7">
         <f t="shared" si="1"/>
-        <v>8166.1499588477345</v>
+        <v>7886.8312757201647</v>
       </c>
       <c r="J7">
         <v>6071.2326312903115</v>
       </c>
       <c r="K7">
+        <v>1783.3609890933087</v>
+      </c>
+      <c r="L7">
         <f t="shared" si="2"/>
-        <v>8120.3945700763488</v>
-      </c>
-      <c r="L7">
-        <v>19611.623209876507</v>
+        <v>13231.630176036639</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
@@ -2330,17 +4075,17 @@
       <c r="D8" s="2">
         <v>2764.9176954732511</v>
       </c>
-      <c r="E8" s="2">
-        <v>2443.4156378600819</v>
+      <c r="E8" s="5">
+        <v>4045.6197993210399</v>
       </c>
       <c r="F8">
         <f t="shared" si="0"/>
-        <v>5208.333333333333</v>
+        <v>6810.537494794291</v>
       </c>
       <c r="G8" s="2">
         <v>2764.9176954732511</v>
       </c>
-      <c r="H8" s="4">
+      <c r="H8">
         <v>0</v>
       </c>
       <c r="I8">
@@ -2351,11 +4096,11 @@
         <v>6403.8158313631438</v>
       </c>
       <c r="K8">
+        <v>2291.7630683822417</v>
+      </c>
+      <c r="L8">
         <f t="shared" si="2"/>
-        <v>6924.9120720465389</v>
-      </c>
-      <c r="L8">
-        <v>17168.207572016425</v>
+        <v>9592.7320401467477</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
@@ -2371,32 +4116,32 @@
       <c r="D9" s="2">
         <v>2767.3611111111113</v>
       </c>
-      <c r="E9" s="2">
-        <v>3469.7788065843624</v>
+      <c r="E9" s="5">
+        <v>2402.5977708842929</v>
       </c>
       <c r="F9">
         <f t="shared" si="0"/>
-        <v>6237.1399176954737</v>
+        <v>5169.9588819954042</v>
       </c>
       <c r="G9" s="2">
         <v>2767.3611111111113</v>
       </c>
-      <c r="H9" s="4">
-        <v>0</v>
+      <c r="H9">
+        <v>585.00395061726795</v>
       </c>
       <c r="I9">
         <f t="shared" si="1"/>
-        <v>2767.3611111111113</v>
+        <v>3352.3650617283793</v>
       </c>
       <c r="J9">
         <v>6026.4848889003415</v>
       </c>
       <c r="K9">
+        <v>1221.1055597510699</v>
+      </c>
+      <c r="L9">
         <f t="shared" si="2"/>
-        <v>7135.5671008416712</v>
-      </c>
-      <c r="L9">
-        <v>13698.428765432065</v>
+        <v>6918.6122129747846</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
@@ -2412,32 +4157,32 @@
       <c r="D10" s="2">
         <v>2767.3611111111113</v>
       </c>
-      <c r="E10" s="2">
-        <v>4530.7355967078192</v>
+      <c r="E10" s="5">
+        <v>1957.8353942526392</v>
       </c>
       <c r="F10">
         <f t="shared" si="0"/>
-        <v>7298.0967078189306</v>
+        <v>4725.1965053637505</v>
       </c>
       <c r="G10" s="2">
         <v>2767.3611111111113</v>
       </c>
-      <c r="H10" s="4">
-        <v>0</v>
+      <c r="H10">
+        <v>3000</v>
       </c>
       <c r="I10">
         <f t="shared" si="1"/>
-        <v>2767.3611111111113</v>
+        <v>5767.3611111111113</v>
       </c>
       <c r="J10">
         <v>4479.7985738060161</v>
       </c>
       <c r="K10">
+        <v>1527.8529741982381</v>
+      </c>
+      <c r="L10">
         <f t="shared" si="2"/>
-        <v>9953.8652348545857</v>
-      </c>
-      <c r="L10">
-        <v>9167.6931687242432</v>
+        <v>8206.1747502798789</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
@@ -2453,17 +4198,17 @@
       <c r="D11" s="2">
         <v>2767.3611111111113</v>
       </c>
-      <c r="E11" s="2">
-        <v>865.61213991769546</v>
+      <c r="E11" s="5">
+        <v>384.25882680588074</v>
       </c>
       <c r="F11">
         <f t="shared" si="0"/>
-        <v>3632.9732510288068</v>
+        <v>3151.6199379169921</v>
       </c>
       <c r="G11" s="2">
         <v>2767.3611111111113</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H11">
         <v>0</v>
       </c>
       <c r="I11">
@@ -2474,11 +4219,11 @@
         <v>4284.164832400751</v>
       </c>
       <c r="K11">
+        <v>112.17185609353919</v>
+      </c>
+      <c r="L11">
         <f t="shared" si="2"/>
-        <v>9302.6736534826414</v>
-      </c>
-      <c r="L11">
-        <v>8302.0810288065477</v>
+        <v>6689.3710289902392</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
@@ -2494,17 +4239,17 @@
       <c r="D12" s="2">
         <v>2767.3611111111113</v>
       </c>
-      <c r="E12" s="2">
-        <v>2955.3755144032921</v>
+      <c r="E12" s="5">
+        <v>1188.9143226231608</v>
       </c>
       <c r="F12">
         <f t="shared" si="0"/>
-        <v>5722.7366255144034</v>
+        <v>3956.2754337342722</v>
       </c>
       <c r="G12" s="2">
         <v>2767.3611111111113</v>
       </c>
-      <c r="H12" s="4">
+      <c r="H12">
         <v>0</v>
       </c>
       <c r="I12">
@@ -2515,11 +4260,11 @@
         <v>3874.8158713185621</v>
       </c>
       <c r="K12">
+        <v>213.99630911317672</v>
+      </c>
+      <c r="L12">
         <f t="shared" si="2"/>
-        <v>11150.594407678484</v>
-      </c>
-      <c r="L12">
-        <v>5346.7055144032556</v>
+        <v>5581.9162687827884</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
@@ -2535,17 +4280,17 @@
       <c r="D13" s="2">
         <v>2767.3611111111113</v>
       </c>
-      <c r="E13" s="2">
-        <v>2440.9722222222217</v>
+      <c r="E13" s="5">
+        <v>1166.5803075057843</v>
       </c>
       <c r="F13">
         <f t="shared" si="0"/>
-        <v>5208.333333333333</v>
+        <v>3933.9414186168956</v>
       </c>
       <c r="G13" s="2">
         <v>2767.3611111111113</v>
       </c>
-      <c r="H13" s="4">
+      <c r="H13">
         <v>0</v>
       </c>
       <c r="I13">
@@ -2556,11 +4301,352 @@
         <v>3826.840185484803</v>
       </c>
       <c r="K13">
+        <v>347.87285052829304</v>
+      </c>
+      <c r="L13">
         <f t="shared" si="2"/>
-        <v>12532.087555527012</v>
-      </c>
-      <c r="L13">
-        <v>2905.7332921810339</v>
+        <v>4522.4371944090963</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="E14" s="5">
+        <f>SUM(E2:E13)</f>
+        <v>18917.677294395813</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="F16" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F17">
+        <f>B2*D2+C2*E2</f>
+        <v>10975.336142410484</v>
+      </c>
+      <c r="G17">
+        <f>B2*G2+C2*H2</f>
+        <v>20896.148657136669</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F18">
+        <f t="shared" ref="F18:F28" si="3">B3*D3+C3*E3</f>
+        <v>7724.5691872427979</v>
+      </c>
+      <c r="G18">
+        <f t="shared" ref="G18:G28" si="4">B3*G3+C3*H3</f>
+        <v>7724.5691872427979</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F19">
+        <f t="shared" si="3"/>
+        <v>11654.663925322006</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="4"/>
+        <v>22004.599980274761</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="C20" t="s">
+        <v>19</v>
+      </c>
+      <c r="D20" t="s">
+        <v>20</v>
+      </c>
+      <c r="F20">
+        <f t="shared" si="3"/>
+        <v>9271.525033990607</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="4"/>
+        <v>11832.14136614685</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21">
+        <v>2348425</v>
+      </c>
+      <c r="D21">
+        <v>890831.11158837902</v>
+      </c>
+      <c r="F21">
+        <f t="shared" si="3"/>
+        <v>9271.525033990607</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="4"/>
+        <v>14421.656662876299</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22">
+        <v>2348425</v>
+      </c>
+      <c r="D22">
+        <v>659262.465350062</v>
+      </c>
+      <c r="F22">
+        <f t="shared" si="3"/>
+        <v>7935.0887345679021</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="4"/>
+        <v>8909.358471410007</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F23">
+        <f t="shared" si="3"/>
+        <v>11727.428796849965</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="4"/>
+        <v>4761.0596707818931</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F24">
+        <f t="shared" si="3"/>
+        <v>8894.5684153182701</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="4"/>
+        <v>5767.5198343467655</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F25">
+        <f t="shared" si="3"/>
+        <v>9252.1442773526396</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="4"/>
+        <v>11642.768858011783</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F26">
+        <f t="shared" si="3"/>
+        <v>4871.2401171827014</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="4"/>
+        <v>4761.0596707818931</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F27">
+        <f t="shared" si="3"/>
+        <v>6465.590096192388</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="4"/>
+        <v>4761.0596707818931</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F28">
+        <f t="shared" si="3"/>
+        <v>6099.0707407492309</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="4"/>
+        <v>4761.0596707818931</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E31" t="s">
+        <v>12</v>
+      </c>
+      <c r="F31">
+        <f>SUM(F17:F28)</f>
+        <v>104142.75050116959</v>
+      </c>
+      <c r="G31">
+        <f>SUM(G17:G28)</f>
+        <v>122243.0017005735</v>
+      </c>
+      <c r="H31">
+        <f>100*(F31-G31)/F31</f>
+        <v>-17.380231568975731</v>
+      </c>
+    </row>
+    <row r="32" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E32" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32">
+        <f>SUM(K2:K13)</f>
+        <v>24428.025380760773</v>
+      </c>
+      <c r="G32">
+        <f>SUM(L2:L13)</f>
+        <v>82362.014998374056</v>
+      </c>
+      <c r="H32">
+        <f t="shared" ref="H32:H34" si="5">100*(F32-G32)/F32</f>
+        <v>-237.16198388774157</v>
+      </c>
+    </row>
+    <row r="33" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
+      </c>
+      <c r="G33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E34" t="s">
+        <v>15</v>
+      </c>
+      <c r="F34">
+        <f>SUM(F31:F33)</f>
+        <v>128570.77588193037</v>
+      </c>
+      <c r="G34">
+        <f>SUM(G31:G33)</f>
+        <v>204605.01669894755</v>
+      </c>
+      <c r="H34">
+        <f t="shared" si="5"/>
+        <v>-59.138043070410689</v>
+      </c>
+    </row>
+    <row r="37" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F37">
+        <f>F31/2.5</f>
+        <v>41657.100200467838</v>
+      </c>
+      <c r="G37">
+        <f>G31/2.5</f>
+        <v>48897.200680229398</v>
+      </c>
+      <c r="H37">
+        <f>100*(F37-G37)/F37</f>
+        <v>-17.380231568975724</v>
+      </c>
+    </row>
+    <row r="38" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F38">
+        <f t="shared" ref="F38:G38" si="6">F32/2.5</f>
+        <v>9771.2101523043093</v>
+      </c>
+      <c r="G38">
+        <f t="shared" si="6"/>
+        <v>32944.805999349621</v>
+      </c>
+      <c r="H38">
+        <f t="shared" ref="H38:H40" si="7">100*(F38-G38)/F38</f>
+        <v>-237.16198388774157</v>
+      </c>
+    </row>
+    <row r="39" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F39">
+        <f t="shared" ref="F39:G39" si="8">F33/2.5</f>
+        <v>0</v>
+      </c>
+      <c r="G39">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F40">
+        <f t="shared" ref="F40:G40" si="9">F34/2.5</f>
+        <v>51428.310352772147</v>
+      </c>
+      <c r="G40">
+        <f t="shared" si="9"/>
+        <v>81842.006679579019</v>
+      </c>
+      <c r="H40">
+        <f t="shared" si="7"/>
+        <v>-59.138043070410689</v>
+      </c>
+    </row>
+    <row r="42" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E42" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="43" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E43" t="s">
+        <v>12</v>
+      </c>
+      <c r="F43">
+        <v>3276</v>
+      </c>
+      <c r="G43">
+        <f>F43*(1-H37/100)</f>
+        <v>3845.3763861996449</v>
+      </c>
+      <c r="H43">
+        <f>F43-G43</f>
+        <v>-569.37638619964491</v>
+      </c>
+    </row>
+    <row r="44" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E44" t="s">
+        <v>13</v>
+      </c>
+      <c r="F44">
+        <v>24.705120059999999</v>
+      </c>
+      <c r="G44">
+        <f>F44*(1-H38/100)</f>
+        <v>83.296272916144417</v>
+      </c>
+      <c r="H44">
+        <f t="shared" ref="H44:H45" si="10">F44-G44</f>
+        <v>-58.591152856144419</v>
+      </c>
+    </row>
+    <row r="45" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45">
+        <v>0</v>
+      </c>
+      <c r="G45">
+        <f>F45*(1-H39/100)</f>
+        <v>0</v>
+      </c>
+      <c r="H45">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E46" t="s">
+        <v>15</v>
+      </c>
+      <c r="F46">
+        <v>3300.7051200000001</v>
+      </c>
+      <c r="G46">
+        <f>SUM(G43:G45)</f>
+        <v>3928.6726591157894</v>
+      </c>
+      <c r="H46">
+        <f>SUM(H43:H45)</f>
+        <v>-627.9675390557893</v>
       </c>
     </row>
   </sheetData>
@@ -2569,9 +4655,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42DA7594-E291-8048-9A99-303698ABB733}">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="12.6640625" customWidth="1"/>
@@ -2636,10 +4722,10 @@
         <f>SUM(D2:E2)</f>
         <v>14400</v>
       </c>
-      <c r="G2" s="2">
-        <v>4886.8312757201647</v>
-      </c>
-      <c r="H2" s="4">
+      <c r="G2" s="6">
+        <v>4886.8312757201647</v>
+      </c>
+      <c r="H2">
         <v>9513.1687242798362</v>
       </c>
       <c r="I2">
@@ -2653,7 +4739,8 @@
         <v>5085.7142857142862</v>
       </c>
       <c r="L2">
-        <v>2113.1687242798344</v>
+        <f>I2-J2</f>
+        <v>4085.7142857142862</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
@@ -2676,15 +4763,15 @@
         <f t="shared" ref="F3:F13" si="0">SUM(D3:E3)</f>
         <v>7457.1428571428569</v>
       </c>
-      <c r="G3" s="2">
-        <v>4886.8312757201647</v>
-      </c>
-      <c r="H3" s="4">
+      <c r="G3" s="6">
+        <v>4886.8312757201647</v>
+      </c>
+      <c r="H3">
         <v>2570.3115814226921</v>
       </c>
-      <c r="I3">
-        <f t="shared" ref="I3:I13" si="1">SUM(G3:H3)</f>
-        <v>7457.1428571428569</v>
+      <c r="I3" s="6">
+        <f>SUM(G3:H3)+1000</f>
+        <v>8457.1428571428569</v>
       </c>
       <c r="J3" s="4">
         <v>12000</v>
@@ -2693,7 +4780,8 @@
         <v>542.85714285714312</v>
       </c>
       <c r="L3">
-        <v>8920.2674897119323</v>
+        <f>L2+I3-J3</f>
+        <v>542.85714285714312</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
@@ -2716,14 +4804,14 @@
         <f t="shared" si="0"/>
         <v>14514.285714285714</v>
       </c>
-      <c r="G4" s="2">
-        <v>4886.8312757201647</v>
-      </c>
-      <c r="H4" s="4">
+      <c r="G4" s="6">
+        <v>4886.8312757201647</v>
+      </c>
+      <c r="H4">
         <v>9627.4544385655499</v>
       </c>
       <c r="I4">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="I4:I13" si="1">SUM(G4:H4)</f>
         <v>14514.285714285714</v>
       </c>
       <c r="J4" s="4">
@@ -2733,7 +4821,8 @@
         <v>5228.5714285714275</v>
       </c>
       <c r="L4">
-        <v>10904.835390946499</v>
+        <f t="shared" ref="L4:L13" si="2">L3+I4-J4</f>
+        <v>5228.5714285714275</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -2756,10 +4845,10 @@
         <f t="shared" si="0"/>
         <v>12228.571428571429</v>
       </c>
-      <c r="G5" s="2">
-        <v>4886.8312757201647</v>
-      </c>
-      <c r="H5" s="4">
+      <c r="G5" s="6">
+        <v>4886.8312757201647</v>
+      </c>
+      <c r="H5">
         <v>7341.7401528512646</v>
       </c>
       <c r="I5">
@@ -2773,7 +4862,8 @@
         <v>4999.9999999999982</v>
       </c>
       <c r="L5">
-        <v>14464.763374485594</v>
+        <f t="shared" si="2"/>
+        <v>4999.9999999999982</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
@@ -2796,15 +4886,15 @@
         <f t="shared" si="0"/>
         <v>12228.571428571429</v>
       </c>
-      <c r="G6" s="2">
-        <v>4886.8312757201647</v>
-      </c>
-      <c r="H6" s="4">
-        <v>15000</v>
+      <c r="G6" s="6">
+        <v>4886.8312757201647</v>
+      </c>
+      <c r="H6">
+        <v>2770.3115821323399</v>
       </c>
       <c r="I6">
         <f t="shared" si="1"/>
-        <v>19886.831275720164</v>
+        <v>7657.1428578525047</v>
       </c>
       <c r="J6" s="4">
         <v>12657.142857142857</v>
@@ -2813,7 +4903,8 @@
         <v>4571.4285714285706</v>
       </c>
       <c r="L6">
-        <v>17682.613168724245</v>
+        <f t="shared" si="2"/>
+        <v>7.0964597398415208E-7</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
@@ -2836,15 +4927,15 @@
         <f t="shared" si="0"/>
         <v>9342.8571428571431</v>
       </c>
-      <c r="G7" s="2">
-        <v>4886.8312757201647</v>
-      </c>
-      <c r="H7" s="4">
-        <v>15000</v>
+      <c r="G7" s="6">
+        <v>4886.8312757201647</v>
+      </c>
+      <c r="H7">
+        <v>7113.1687252683996</v>
       </c>
       <c r="I7">
         <f t="shared" si="1"/>
-        <v>19886.831275720164</v>
+        <v>12000.000000988564</v>
       </c>
       <c r="J7" s="4">
         <v>12000</v>
@@ -2853,7 +4944,8 @@
         <v>1914.2857142857138</v>
       </c>
       <c r="L7">
-        <v>19611.623209876507</v>
+        <f t="shared" si="2"/>
+        <v>1.6982103261398152E-6</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
@@ -2876,15 +4968,15 @@
         <f t="shared" si="0"/>
         <v>13314.285714285714</v>
       </c>
-      <c r="G8" s="2">
-        <v>2767.3611111111113</v>
-      </c>
-      <c r="H8" s="4">
-        <v>15000</v>
+      <c r="G8" s="6">
+        <v>2767.3611111111113</v>
+      </c>
+      <c r="H8">
+        <v>8946.9245985163598</v>
       </c>
       <c r="I8">
         <f t="shared" si="1"/>
-        <v>17767.361111111109</v>
+        <v>11714.285709627471</v>
       </c>
       <c r="J8" s="4">
         <v>11714.285714285714</v>
@@ -2893,7 +4985,8 @@
         <v>3514.2857142857138</v>
       </c>
       <c r="L8">
-        <v>17168.207572016425</v>
+        <f t="shared" si="2"/>
+        <v>-2.9600323614431545E-6</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
@@ -2916,15 +5009,15 @@
         <f t="shared" si="0"/>
         <v>10114.285714285714</v>
       </c>
-      <c r="G9" s="2">
-        <v>2767.3611111111113</v>
-      </c>
-      <c r="H9" s="4">
-        <v>3088.8718871251899</v>
+      <c r="G9" s="6">
+        <v>2767.3611111111113</v>
+      </c>
+      <c r="H9">
+        <v>6575.4960321757098</v>
       </c>
       <c r="I9">
         <f t="shared" si="1"/>
-        <v>5856.2329982363008</v>
+        <v>9342.8571432868212</v>
       </c>
       <c r="J9" s="4">
         <v>9342.8571428571431</v>
@@ -2933,7 +5026,8 @@
         <v>4285.7142857142844</v>
       </c>
       <c r="L9">
-        <v>13698.428765432065</v>
+        <f t="shared" si="2"/>
+        <v>-2.5303543225163594E-6</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
@@ -2956,15 +5050,15 @@
         <f t="shared" si="0"/>
         <v>9228.5714285714294</v>
       </c>
-      <c r="G10" s="2">
-        <v>2767.3611111111113</v>
-      </c>
-      <c r="H10" s="4">
-        <v>0</v>
+      <c r="G10" s="6">
+        <v>2767.3611111111113</v>
+      </c>
+      <c r="H10">
+        <v>6318.3531745687897</v>
       </c>
       <c r="I10">
         <f t="shared" si="1"/>
-        <v>2767.3611111111113</v>
+        <v>9085.7142856799001</v>
       </c>
       <c r="J10" s="4">
         <v>9085.7142857142862</v>
@@ -2973,7 +5067,8 @@
         <v>4428.5714285714275</v>
       </c>
       <c r="L10">
-        <v>9167.6931687242432</v>
+        <f t="shared" si="2"/>
+        <v>-2.5647404982009903E-6</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
@@ -2996,15 +5091,15 @@
         <f t="shared" si="0"/>
         <v>6171.4285714285716</v>
       </c>
-      <c r="G11" s="2">
-        <v>2767.3611111111113</v>
-      </c>
-      <c r="H11" s="4">
-        <v>0</v>
+      <c r="G11" s="6">
+        <v>2767.3611111111113</v>
+      </c>
+      <c r="H11">
+        <v>6261.2103190224898</v>
       </c>
       <c r="I11">
         <f t="shared" si="1"/>
-        <v>2767.3611111111113</v>
+        <v>9028.5714301336011</v>
       </c>
       <c r="J11" s="4">
         <v>9028.5714285714294</v>
@@ -3013,7 +5108,8 @@
         <v>1571.4285714285706</v>
       </c>
       <c r="L11">
-        <v>8302.0810288065477</v>
+        <f t="shared" si="2"/>
+        <v>-1.0025687515735626E-6</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
@@ -3036,15 +5132,15 @@
         <f t="shared" si="0"/>
         <v>7742.8571428571431</v>
       </c>
-      <c r="G12" s="2">
-        <v>2767.3611111111113</v>
-      </c>
-      <c r="H12" s="4">
-        <v>0</v>
+      <c r="G12" s="6">
+        <v>2767.3611111111113</v>
+      </c>
+      <c r="H12">
+        <v>4918.3531744415704</v>
       </c>
       <c r="I12">
         <f t="shared" si="1"/>
-        <v>2767.3611111111113</v>
+        <v>7685.7142855526818</v>
       </c>
       <c r="J12" s="4">
         <v>7685.7142857142853</v>
@@ -3053,7 +5149,8 @@
         <v>1628.5714285714284</v>
       </c>
       <c r="L12">
-        <v>5346.7055144032556</v>
+        <f t="shared" si="2"/>
+        <v>-1.1641723176580854E-6</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
@@ -3076,15 +5173,15 @@
         <f t="shared" si="0"/>
         <v>7685.7142857142853</v>
       </c>
-      <c r="G13" s="2">
-        <v>2767.3611111111113</v>
-      </c>
-      <c r="H13" s="4">
-        <v>0</v>
+      <c r="G13" s="6">
+        <v>2767.3611111111113</v>
+      </c>
+      <c r="H13">
+        <v>4804.0674598933701</v>
       </c>
       <c r="I13">
         <f t="shared" si="1"/>
-        <v>2767.3611111111113</v>
+        <v>7571.4285710044815</v>
       </c>
       <c r="J13" s="4">
         <v>7571.4285714285716</v>
@@ -3093,7 +5190,262 @@
         <v>1742.8571428571422</v>
       </c>
       <c r="L13">
-        <v>2905.7332921810339</v>
+        <f t="shared" si="2"/>
+        <v>-1.5882624211371876E-6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="F16" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F17">
+        <f>B2*D2+C2*E2</f>
+        <v>20896.148657136669</v>
+      </c>
+      <c r="G17">
+        <f>B2*G2+C2*H2</f>
+        <v>20896.148657136669</v>
+      </c>
+    </row>
+    <row r="18" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F18">
+        <f t="shared" ref="F18:F28" si="3">B3*D3+C3*E3</f>
+        <v>7724.5691872427979</v>
+      </c>
+      <c r="G18">
+        <f t="shared" ref="G18:G28" si="4">B3*G3+C3*H3</f>
+        <v>7724.5691872427979</v>
+      </c>
+    </row>
+    <row r="19" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F19">
+        <f t="shared" si="3"/>
+        <v>22004.599980274761</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="4"/>
+        <v>22004.599980274761</v>
+      </c>
+    </row>
+    <row r="20" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F20">
+        <f t="shared" si="3"/>
+        <v>15087.875680327363</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="4"/>
+        <v>15087.875680327363</v>
+      </c>
+    </row>
+    <row r="21" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F21">
+        <f t="shared" si="3"/>
+        <v>15087.875680327363</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="4"/>
+        <v>10634.101244928521</v>
+      </c>
+    </row>
+    <row r="22" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F22">
+        <f t="shared" si="3"/>
+        <v>9382.2124508802881</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="4"/>
+        <v>10245.137075261482</v>
+      </c>
+    </row>
+    <row r="23" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F23">
+        <f t="shared" si="3"/>
+        <v>22926.580730897007</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="4"/>
+        <v>20171.455141480383</v>
+      </c>
+    </row>
+    <row r="24" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F24">
+        <f t="shared" si="3"/>
+        <v>17400.951982633287</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="4"/>
+        <v>16073.760730459811</v>
+      </c>
+    </row>
+    <row r="25" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F25">
+        <f t="shared" si="3"/>
+        <v>19582.449804878968</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="4"/>
+        <v>19254.74936731295</v>
+      </c>
+    </row>
+    <row r="26" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F26">
+        <f t="shared" si="3"/>
+        <v>5737.1248804581701</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="4"/>
+        <v>6556.3676763094973</v>
+      </c>
+    </row>
+    <row r="27" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F27">
+        <f t="shared" si="3"/>
+        <v>11894.361210045459</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="4"/>
+        <v>11812.436266408275</v>
+      </c>
+    </row>
+    <row r="28" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="F28">
+        <f t="shared" si="3"/>
+        <v>10402.172375399885</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="4"/>
+        <v>10271.092199918621</v>
+      </c>
+    </row>
+    <row r="31" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E31" t="s">
+        <v>12</v>
+      </c>
+      <c r="F31">
+        <f>SUM(F17:F28)</f>
+        <v>178126.92262050201</v>
+      </c>
+      <c r="G31">
+        <f>SUM(G17:G28)</f>
+        <v>170732.29320706113</v>
+      </c>
+      <c r="H31">
+        <f>100*(F31-G31)/F31</f>
+        <v>4.1513260907757781</v>
+      </c>
+    </row>
+    <row r="32" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E32" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32">
+        <f>0.05*SUM(K2:K13)</f>
+        <v>1975.7142857142856</v>
+      </c>
+      <c r="G32">
+        <f>0.05*SUM(L2:L13)</f>
+        <v>742.85714238702917</v>
+      </c>
+      <c r="H32">
+        <f t="shared" ref="H32:H34" si="5">100*(F32-G32)/F32</f>
+        <v>62.400578476433807</v>
+      </c>
+    </row>
+    <row r="33" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
+      </c>
+      <c r="G33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E34" t="s">
+        <v>15</v>
+      </c>
+      <c r="F34">
+        <f>SUM(F31:F33)</f>
+        <v>180102.6369062163</v>
+      </c>
+      <c r="G34">
+        <f>SUM(G31:G33)</f>
+        <v>171475.15034944814</v>
+      </c>
+      <c r="H34">
+        <f t="shared" si="5"/>
+        <v>4.7903166244371489</v>
+      </c>
+    </row>
+    <row r="37" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E37" t="s">
+        <v>12</v>
+      </c>
+      <c r="F37">
+        <v>2768</v>
+      </c>
+      <c r="G37">
+        <f>F37*(1-H31/100)</f>
+        <v>2653.0912938073266</v>
+      </c>
+      <c r="H37">
+        <f>F37-G37</f>
+        <v>114.90870619267343</v>
+      </c>
+    </row>
+    <row r="38" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E38" t="s">
+        <v>13</v>
+      </c>
+      <c r="F38">
+        <v>30.7</v>
+      </c>
+      <c r="G38">
+        <f>F38*(1-H32/100)</f>
+        <v>11.543022407734821</v>
+      </c>
+      <c r="H38">
+        <f t="shared" ref="H38:H39" si="6">F38-G38</f>
+        <v>19.156977592265179</v>
+      </c>
+    </row>
+    <row r="39" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E39" t="s">
+        <v>14</v>
+      </c>
+      <c r="F39">
+        <v>0</v>
+      </c>
+      <c r="G39">
+        <f>F39*(1-H33/100)</f>
+        <v>0</v>
+      </c>
+      <c r="H39">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="5:8" x14ac:dyDescent="0.2">
+      <c r="E40" t="s">
+        <v>15</v>
+      </c>
+      <c r="F40">
+        <v>2798.7</v>
+      </c>
+      <c r="G40">
+        <f>SUM(G37:G39)</f>
+        <v>2664.6343162150615</v>
+      </c>
+      <c r="H40">
+        <f>SUM(H37:H39)</f>
+        <v>134.06568378493861</v>
       </c>
     </row>
   </sheetData>

</xml_diff>